<commit_message>
update initial guesses for height difference
</commit_message>
<xml_diff>
--- a/script/simulation_queue_example.xlsx
+++ b/script/simulation_queue_example.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f03addda2663411/SRBL/WearableOptimizedControl/Optimizer/Moco_git/script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="124" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E4DEB7E1-A8E7-415C-BC10-CA8E1DBD4434}"/>
+  <xr:revisionPtr revIDLastSave="134" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B3EB3C53-59A5-4573-953A-7EBE4B6CF966}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="simulation_queue" sheetId="1" r:id="rId1"/>
     <sheet name="completed_queue" sheetId="2" r:id="rId2"/>
     <sheet name="models" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="484" uniqueCount="112">
   <si>
     <t>SF</t>
   </si>
@@ -411,12 +411,20 @@
     <t>2D_gait_AFO_pc_v38.osim</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
+  <si>
+    <t>2D_gait_AFO_pc_50BW.osim</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
+  <si>
+    <t>test1</t>
+    <phoneticPr fontId="18" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -626,19 +634,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79995117038483843"/>
+        <fgColor theme="4" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59996337778862885"/>
+        <fgColor theme="4" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -649,19 +657,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79995117038483843"/>
+        <fgColor theme="5" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59996337778862885"/>
+        <fgColor theme="5" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -672,19 +680,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79995117038483843"/>
+        <fgColor theme="6" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59996337778862885"/>
+        <fgColor theme="6" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="6" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -695,19 +703,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79995117038483843"/>
+        <fgColor theme="7" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59996337778862885"/>
+        <fgColor theme="7" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -718,19 +726,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79995117038483843"/>
+        <fgColor theme="8" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59996337778862885"/>
+        <fgColor theme="8" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -741,24 +749,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79995117038483843"/>
+        <fgColor theme="9" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59996337778862885"/>
+        <fgColor theme="9" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -780,7 +788,7 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.49995422223578601"/>
+        <color theme="4" tint="0.49995422223579"/>
       </bottom>
       <diagonal/>
     </border>
@@ -789,7 +797,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
+        <color theme="4" tint="0.39997558519242"/>
       </bottom>
       <diagonal/>
     </border>
@@ -873,191 +881,193 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="false" applyFont="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="true"/>
+    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="true"/>
+    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="true"/>
+    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="true"/>
+    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="true"/>
+    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="true"/>
+    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="true"/>
+    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="true"/>
+    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="true"/>
+    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="true"/>
+    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="true"/>
+    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="true"/>
+    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="true"/>
+    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="true"/>
+    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="true"/>
+    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="true"/>
+    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="true"/>
+    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="true"/>
+    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="true"/>
+    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="true"/>
+    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="true"/>
+    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="true"/>
+    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="true"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1074,7 +1084,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1225,7 +1235,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1249,9 +1259,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1275,7 +1285,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1310,7 +1320,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1328,7 +1338,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1353,7 +1363,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1369,391 +1379,663 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U16"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U17"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.75" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="6.625" customWidth="1"/>
-    <col min="4" max="4" width="4" customWidth="1"/>
-    <col min="5" max="5" width="13.5" customWidth="1"/>
-    <col min="6" max="6" width="6.875" customWidth="1"/>
-    <col min="7" max="7" width="4.125" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="3.875" customWidth="1"/>
-    <col min="10" max="10" width="7.5" customWidth="1"/>
-    <col min="11" max="11" width="11.375" customWidth="1"/>
-    <col min="12" max="12" width="9.25" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="4.625" customWidth="1"/>
-    <col min="15" max="15" width="10.625" customWidth="1"/>
-    <col min="16" max="16" width="14.125" customWidth="1"/>
-    <col min="17" max="17" width="15.75" customWidth="1"/>
-    <col min="18" max="18" width="14.875" customWidth="1"/>
-    <col min="19" max="19" width="9.5" customWidth="1"/>
-    <col min="20" max="20" width="12.875" customWidth="1"/>
-    <col min="21" max="21" width="9.5" customWidth="1"/>
+    <col min="1" max="1" width="25.75" customWidth="true"/>
+    <col min="2" max="2" width="10" customWidth="true"/>
+    <col min="3" max="3" width="22.75" customWidth="true"/>
+    <col min="4" max="4" width="4" customWidth="true"/>
+    <col min="5" max="5" width="13.5" customWidth="true"/>
+    <col min="6" max="6" width="6.875" customWidth="true"/>
+    <col min="7" max="7" width="4.125" customWidth="true"/>
+    <col min="8" max="8" width="4" customWidth="true"/>
+    <col min="9" max="9" width="3.875" customWidth="true"/>
+    <col min="10" max="10" width="7.5" customWidth="true"/>
+    <col min="11" max="11" width="14.375" customWidth="true"/>
+    <col min="12" max="12" width="9.25" customWidth="true"/>
+    <col min="13" max="13" width="11" customWidth="true"/>
+    <col min="14" max="14" width="4.625" customWidth="true"/>
+    <col min="15" max="15" width="10.625" customWidth="true"/>
+    <col min="16" max="16" width="14.125" customWidth="true"/>
+    <col min="17" max="17" width="15.75" customWidth="true"/>
+    <col min="18" max="18" width="14.875" customWidth="true"/>
+    <col min="19" max="19" width="10.625" customWidth="true"/>
+    <col min="20" max="20" width="12.875" customWidth="true"/>
+    <col min="21" max="21" width="9.5" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="2">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="K2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="0"/>
+      <c r="P2" s="0"/>
+      <c r="Q2" s="0"/>
+      <c r="R2" s="0"/>
+      <c r="S2" s="0"/>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="K3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="0"/>
+      <c r="P3" s="0"/>
+      <c r="Q3" s="0"/>
+      <c r="R3" s="0"/>
+      <c r="S3" s="0"/>
+      <c r="T3" s="0"/>
+      <c r="U3" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="2">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+        <v>0.029999999999999999</v>
+      </c>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="0"/>
+      <c r="P4" s="0"/>
+      <c r="Q4" s="0"/>
+      <c r="R4" s="0"/>
+      <c r="S4" s="0"/>
+      <c r="T4" s="0"/>
+      <c r="U4" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0"/>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0"/>
+      <c r="T5" s="0"/>
+      <c r="U5" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="0"/>
+      <c r="P6" s="0"/>
+      <c r="Q6" s="0"/>
+      <c r="R6" s="0"/>
+      <c r="S6" s="0"/>
+      <c r="T6" s="0"/>
+      <c r="U6" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" ht="165" x14ac:dyDescent="0.3">
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+      <c r="S7" s="0"/>
+      <c r="T7" s="0"/>
+      <c r="U7" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" ht="165" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+      <c r="S8" s="0"/>
+      <c r="T8" s="0"/>
+      <c r="U8" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C9" s="0"/>
+      <c r="D9" s="0"/>
+      <c r="E9" s="0"/>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
+      <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
+      <c r="K9" s="0"/>
+      <c r="L9" s="0"/>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+      <c r="O9" s="0"/>
+      <c r="P9" s="0"/>
+      <c r="Q9" s="0"/>
+      <c r="R9" s="0"/>
+      <c r="S9" s="0"/>
+      <c r="T9" s="0"/>
+      <c r="U9" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N10" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="O10" t="s">
+      <c r="O10" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="Q10" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="S10" t="s">
+      <c r="S10" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="T10" t="s">
+      <c r="T10" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="U10" t="s">
+      <c r="U10" s="0" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+      <c r="A11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="0">
         <v>260515</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>3</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K11" t="s">
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
+      <c r="K11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="O11">
-        <v>1</v>
-      </c>
-      <c r="P11">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0">
+        <v>0.010999999999999999</v>
+      </c>
+      <c r="Q11" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U11">
+      <c r="T11" s="0"/>
+      <c r="U11" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+      <c r="A12" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="0">
         <v>260515</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="0">
         <v>3</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K12" t="s">
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
+      <c r="K12" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="O12">
-        <v>1</v>
-      </c>
-      <c r="P12">
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0">
+        <v>1</v>
+      </c>
+      <c r="P12" s="0">
         <v>0.70099999999999996</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="Q12" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S12" t="s">
+      <c r="S12" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U12">
+      <c r="T12" s="0"/>
+      <c r="U12" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+      <c r="A13" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="0">
         <v>260515</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K13" t="s">
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="K13" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="O13">
-        <v>1</v>
-      </c>
-      <c r="P13">
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="0">
+        <v>1</v>
+      </c>
+      <c r="P13" s="0">
         <v>0.10100000000000001</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="Q13" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R13" t="s">
+      <c r="R13" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S13" t="s">
+      <c r="S13" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U13">
+      <c r="T13" s="0"/>
+      <c r="U13" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+      <c r="A14" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="0">
         <v>260515</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="0">
         <v>3</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K14" t="s">
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="K14" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="O14">
-        <v>1</v>
-      </c>
-      <c r="P14">
-        <v>5.0999999999999997E-2</v>
-      </c>
-      <c r="Q14" t="s">
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="0">
+        <v>1</v>
+      </c>
+      <c r="P14" s="0">
+        <v>0.050999999999999997</v>
+      </c>
+      <c r="Q14" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S14" t="s">
+      <c r="S14" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U14">
+      <c r="T14" s="0"/>
+      <c r="U14" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="0">
         <v>260515</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="0">
         <v>3</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K15" t="s">
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="O15">
-        <v>1</v>
-      </c>
-      <c r="P15">
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0">
+        <v>1</v>
+      </c>
+      <c r="P15" s="0">
         <v>1.0049999999999999</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="Q15" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R15" t="s">
+      <c r="R15" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S15" t="s">
+      <c r="S15" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U15">
+      <c r="T15" s="0"/>
+      <c r="U15" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+      <c r="A16" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="0">
         <v>260515</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="0">
         <v>3</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K16" t="s">
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="O16">
-        <v>1</v>
-      </c>
-      <c r="P16">
+      <c r="L16" s="0"/>
+      <c r="M16" s="0"/>
+      <c r="N16" s="0"/>
+      <c r="O16" s="0">
+        <v>1</v>
+      </c>
+      <c r="P16" s="0">
         <v>2.0049999999999999</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="Q16" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U16">
+      <c r="T16" s="0"/>
+      <c r="U16" s="0">
+        <v>-1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+      <c r="A17" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="B17" s="0">
+        <v>260605</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="0">
+        <v>3</v>
+      </c>
+      <c r="E17" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
+      <c r="K17" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="L17" s="0"/>
+      <c r="M17" s="0"/>
+      <c r="N17" s="0"/>
+      <c r="O17" s="0">
+        <v>1</v>
+      </c>
+      <c r="P17" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q17" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="R17" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="S17" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="T17" s="0"/>
+      <c r="U17" s="0">
         <v>-1</v>
       </c>
     </row>
@@ -1765,686 +2047,944 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
   <dimension ref="A1:U22"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.375" customWidth="1"/>
-    <col min="2" max="2" width="7.25" customWidth="1"/>
-    <col min="3" max="3" width="19.125" customWidth="1"/>
-    <col min="4" max="4" width="4" customWidth="1"/>
-    <col min="5" max="5" width="13.5" customWidth="1"/>
-    <col min="6" max="6" width="6.875" customWidth="1"/>
-    <col min="7" max="7" width="4.125" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="3.875" customWidth="1"/>
-    <col min="10" max="10" width="7.5" customWidth="1"/>
-    <col min="11" max="11" width="11.375" customWidth="1"/>
-    <col min="12" max="12" width="9.25" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="4.625" customWidth="1"/>
-    <col min="15" max="15" width="10.625" customWidth="1"/>
-    <col min="16" max="16" width="14.125" customWidth="1"/>
-    <col min="17" max="17" width="15.75" customWidth="1"/>
-    <col min="18" max="18" width="14.875" customWidth="1"/>
-    <col min="19" max="19" width="9.625" customWidth="1"/>
-    <col min="20" max="20" width="12.875" customWidth="1"/>
-    <col min="21" max="21" width="9.5" customWidth="1"/>
+    <col min="1" max="1" width="10.375" customWidth="true"/>
+    <col min="2" max="2" width="7.25" customWidth="true"/>
+    <col min="3" max="3" width="24.75" customWidth="true"/>
+    <col min="4" max="4" width="4" customWidth="true"/>
+    <col min="5" max="5" width="13.5" customWidth="true"/>
+    <col min="6" max="6" width="6.875" customWidth="true"/>
+    <col min="7" max="7" width="4.125" customWidth="true"/>
+    <col min="8" max="8" width="4" customWidth="true"/>
+    <col min="9" max="9" width="3.875" customWidth="true"/>
+    <col min="10" max="10" width="7.5" customWidth="true"/>
+    <col min="11" max="11" width="11.375" customWidth="true"/>
+    <col min="12" max="12" width="9.25" customWidth="true"/>
+    <col min="13" max="13" width="11" customWidth="true"/>
+    <col min="14" max="14" width="4.625" customWidth="true"/>
+    <col min="15" max="15" width="10.625" customWidth="true"/>
+    <col min="16" max="16" width="14.125" customWidth="true"/>
+    <col min="17" max="17" width="15.75" customWidth="true"/>
+    <col min="18" max="18" width="14.875" customWidth="true"/>
+    <col min="19" max="19" width="10.625" customWidth="true"/>
+    <col min="20" max="20" width="12.875" customWidth="true"/>
+    <col min="21" max="21" width="9.5" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
+      <c r="B1" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="K2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="0"/>
+      <c r="P2" s="0"/>
+      <c r="Q2" s="0"/>
+      <c r="R2" s="0"/>
+      <c r="S2" s="0"/>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="K3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="0"/>
+      <c r="P3" s="0"/>
+      <c r="Q3" s="0"/>
+      <c r="R3" s="0"/>
+      <c r="S3" s="0"/>
+      <c r="T3" s="0"/>
+      <c r="U3" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="0"/>
+      <c r="P4" s="0"/>
+      <c r="Q4" s="0"/>
+      <c r="R4" s="0"/>
+      <c r="S4" s="0"/>
+      <c r="T4" s="0"/>
+      <c r="U4" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0"/>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0"/>
+      <c r="T5" s="0"/>
+      <c r="U5" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="0"/>
+      <c r="P6" s="0"/>
+      <c r="Q6" s="0"/>
+      <c r="R6" s="0"/>
+      <c r="S6" s="0"/>
+      <c r="T6" s="0"/>
+      <c r="U6" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B7" s="0">
+        <v>1</v>
+      </c>
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+      <c r="S7" s="0"/>
+      <c r="T7" s="0"/>
+      <c r="U7" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B8" s="0"/>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+      <c r="S8" s="0"/>
+      <c r="T8" s="0"/>
+      <c r="U8" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O9" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="Q9" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="R9" t="s">
+      <c r="R9" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="S9" t="s">
+      <c r="S9" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="T9" t="s">
+      <c r="T9" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="U9" t="s">
+      <c r="U9" s="0" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+      <c r="A10" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="0">
         <v>260501</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="0">
         <v>3</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F10">
-        <v>0.2</v>
-      </c>
-      <c r="G10">
-        <v>0.3</v>
-      </c>
-      <c r="H10">
+      <c r="F10" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G10" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H10" s="0">
         <v>0</v>
       </c>
-      <c r="I10">
-        <v>0.1</v>
-      </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="I10" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J10" s="0">
+        <v>1</v>
+      </c>
+      <c r="K10" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="O10">
-        <v>1</v>
-      </c>
-      <c r="P10">
-        <v>1E-4</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="L10" s="0"/>
+      <c r="M10" s="0"/>
+      <c r="N10" s="0"/>
+      <c r="O10" s="0">
+        <v>1</v>
+      </c>
+      <c r="P10" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q10" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S10" t="s">
+      <c r="S10" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="T10" s="0"/>
+      <c r="U10" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+      <c r="A11" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="0">
         <v>260501</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>3</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F11">
-        <v>0.2</v>
-      </c>
-      <c r="G11">
-        <v>0.3</v>
-      </c>
-      <c r="H11">
+      <c r="F11" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G11" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H11" s="0">
         <v>0</v>
       </c>
-      <c r="I11">
-        <v>0.1</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="I11" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J11" s="0">
+        <v>1</v>
+      </c>
+      <c r="K11" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="O11">
-        <v>1</v>
-      </c>
-      <c r="P11">
-        <v>1E-4</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q11" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="T11" s="0"/>
+      <c r="U11" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+      <c r="A12" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="0">
         <v>260501</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="0">
         <v>3</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F12">
-        <v>0.2</v>
-      </c>
-      <c r="G12">
-        <v>0.3</v>
-      </c>
-      <c r="H12">
+      <c r="F12" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G12" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H12" s="0">
         <v>0</v>
       </c>
-      <c r="I12">
-        <v>0.1</v>
-      </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="I12" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J12" s="0">
+        <v>1</v>
+      </c>
+      <c r="K12" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="O12">
-        <v>1</v>
-      </c>
-      <c r="P12">
-        <v>1E-4</v>
-      </c>
-      <c r="Q12" t="s">
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0">
+        <v>1</v>
+      </c>
+      <c r="P12" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q12" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S12" t="s">
+      <c r="S12" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="T12" s="0"/>
+      <c r="U12" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+      <c r="A13" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="0">
         <v>260513</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K13" t="s">
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="K13" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="S13" t="s">
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="0"/>
+      <c r="P13" s="0"/>
+      <c r="Q13" s="0"/>
+      <c r="R13" s="0"/>
+      <c r="S13" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="T13" s="0"/>
+      <c r="U13" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+      <c r="A14" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="0">
         <v>260513</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="0">
         <v>3</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K14" t="s">
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="K14" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="S14" t="s">
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="0"/>
+      <c r="P14" s="0"/>
+      <c r="Q14" s="0"/>
+      <c r="R14" s="0"/>
+      <c r="S14" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="T14" s="0"/>
+      <c r="U14" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="0">
         <v>260513</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="0">
         <v>3</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K15" t="s">
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="S15" t="s">
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0"/>
+      <c r="P15" s="0"/>
+      <c r="Q15" s="0"/>
+      <c r="R15" s="0"/>
+      <c r="S15" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="T15" s="0"/>
+      <c r="U15" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+      <c r="A16" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="0">
         <v>260419</v>
       </c>
-      <c r="C16" t="s">
-        <v>49</v>
-      </c>
-      <c r="D16">
+      <c r="C16" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D16" s="0">
         <v>3</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K16" t="s">
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="0">
         <v>0.01</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="0">
         <v>0</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O16">
-        <v>1</v>
-      </c>
-      <c r="P16">
-        <v>1E-3</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="O16" s="0">
+        <v>1</v>
+      </c>
+      <c r="P16" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q16" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="T16" s="0"/>
+      <c r="U16" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+      <c r="A17" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="0">
         <v>260419</v>
       </c>
-      <c r="C17" t="s">
-        <v>49</v>
-      </c>
-      <c r="D17">
+      <c r="C17" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D17" s="0">
         <v>3</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K17" t="s">
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
+      <c r="K17" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="0">
         <v>0.01</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="0">
         <v>0</v>
       </c>
-      <c r="N17" t="s">
+      <c r="N17" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O17">
-        <v>1</v>
-      </c>
-      <c r="P17">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="O17" s="0">
+        <v>1</v>
+      </c>
+      <c r="P17" s="0">
+        <v>0.0050000000000000001</v>
+      </c>
+      <c r="Q17" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R17" t="s">
+      <c r="R17" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S17" t="s">
+      <c r="S17" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="T17" s="0"/>
+      <c r="U17" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+      <c r="A18" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="0">
         <v>260419</v>
       </c>
-      <c r="C18" t="s">
-        <v>49</v>
-      </c>
-      <c r="D18">
+      <c r="C18" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="D18" s="0">
         <v>3</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K18" t="s">
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
+      <c r="K18" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="0">
         <v>0.01</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="0">
         <v>0</v>
       </c>
-      <c r="N18" t="s">
+      <c r="N18" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O18">
-        <v>1</v>
-      </c>
-      <c r="P18">
+      <c r="O18" s="0">
+        <v>1</v>
+      </c>
+      <c r="P18" s="0">
         <v>0.01</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="Q18" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R18" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S18" t="s">
+      <c r="S18" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="T18" s="0"/>
+      <c r="U18" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+      <c r="A19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="0">
         <v>260416</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="0">
         <v>3</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K19" t="s">
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
+      <c r="K19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="O19">
-        <v>1</v>
-      </c>
-      <c r="P19">
-        <v>1E-3</v>
-      </c>
-      <c r="Q19" t="s">
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+      <c r="O19" s="0">
+        <v>1</v>
+      </c>
+      <c r="P19" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q19" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R19" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S19" t="s">
+      <c r="S19" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="T19" s="0"/>
+      <c r="U19" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+      <c r="A20" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="0">
         <v>260416</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="0">
         <v>3</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K20" t="s">
+      <c r="F20" s="0"/>
+      <c r="G20" s="0"/>
+      <c r="H20" s="0"/>
+      <c r="I20" s="0"/>
+      <c r="J20" s="0"/>
+      <c r="K20" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="O20">
-        <v>1</v>
-      </c>
-      <c r="P20">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="Q20" t="s">
+      <c r="L20" s="0"/>
+      <c r="M20" s="0"/>
+      <c r="N20" s="0"/>
+      <c r="O20" s="0">
+        <v>1</v>
+      </c>
+      <c r="P20" s="0">
+        <v>0.0050000000000000001</v>
+      </c>
+      <c r="Q20" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R20" t="s">
+      <c r="R20" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S20" t="s">
+      <c r="S20" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="T20" s="0"/>
+      <c r="U20" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+      <c r="A21" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="0">
         <v>260416</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="0">
         <v>3</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K21" t="s">
+      <c r="F21" s="0"/>
+      <c r="G21" s="0"/>
+      <c r="H21" s="0"/>
+      <c r="I21" s="0"/>
+      <c r="J21" s="0"/>
+      <c r="K21" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="O21">
-        <v>1</v>
-      </c>
-      <c r="P21">
+      <c r="L21" s="0"/>
+      <c r="M21" s="0"/>
+      <c r="N21" s="0"/>
+      <c r="O21" s="0">
+        <v>1</v>
+      </c>
+      <c r="P21" s="0">
         <v>0.01</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="Q21" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R21" t="s">
+      <c r="R21" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S21" t="s">
+      <c r="S21" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="T21" s="0"/>
+      <c r="U21" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+      <c r="A22" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="0">
         <v>260416</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="0">
         <v>3</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K22" t="s">
+      <c r="F22" s="0"/>
+      <c r="G22" s="0"/>
+      <c r="H22" s="0"/>
+      <c r="I22" s="0"/>
+      <c r="J22" s="0"/>
+      <c r="K22" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="O22">
-        <v>1</v>
-      </c>
-      <c r="P22">
-        <v>0.03</v>
-      </c>
-      <c r="Q22" t="s">
+      <c r="L22" s="0"/>
+      <c r="M22" s="0"/>
+      <c r="N22" s="0"/>
+      <c r="O22" s="0">
+        <v>1</v>
+      </c>
+      <c r="P22" s="0">
+        <v>0.029999999999999999</v>
+      </c>
+      <c r="Q22" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R22" t="s">
+      <c r="R22" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S22" t="s">
+      <c r="S22" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U22">
+      <c r="T22" s="0"/>
+      <c r="U22" s="0">
         <v>1</v>
       </c>
     </row>
@@ -2456,20 +2996,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.375" customWidth="1"/>
-    <col min="2" max="2" width="24.75" customWidth="1"/>
-    <col min="3" max="3" width="7.25" customWidth="1"/>
-    <col min="4" max="4" width="5.75" customWidth="1"/>
-    <col min="5" max="5" width="6.25" customWidth="1"/>
-    <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="9.375" customWidth="1"/>
+    <col min="1" max="1" width="27.375" customWidth="true"/>
+    <col min="2" max="2" width="24.75" customWidth="true"/>
+    <col min="3" max="3" width="7.25" customWidth="true"/>
+    <col min="4" max="4" width="5.75" customWidth="true"/>
+    <col min="5" max="5" width="6.25" customWidth="true"/>
+    <col min="6" max="6" width="4" customWidth="true"/>
+    <col min="7" max="7" width="9.375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -2477,7 +3017,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -2485,7 +3025,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -2493,12 +3033,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -2521,7 +3061,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -2538,7 +3078,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2555,7 +3095,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -2572,7 +3112,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -2589,7 +3129,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -2606,7 +3146,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -2623,7 +3163,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -2640,7 +3180,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -2657,7 +3197,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -2674,7 +3214,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -2691,7 +3231,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -2708,7 +3248,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -2725,7 +3265,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -2742,7 +3282,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -2759,7 +3299,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -2776,7 +3316,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -2793,7 +3333,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -2810,7 +3350,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -2827,7 +3367,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -2844,7 +3384,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -2861,7 +3401,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>68</v>
       </c>
@@ -2878,7 +3418,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -2895,7 +3435,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -2912,7 +3452,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>71</v>
       </c>
@@ -2929,7 +3469,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>72</v>
       </c>

</xml_diff>

<commit_message>
script 청소 -> legacy 폴더 생성
</commit_message>
<xml_diff>
--- a/script/simulation_queue_example.xlsx
+++ b/script/simulation_queue_example.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f03addda2663411/SRBL/WearableOptimizedControl/Optimizer/Moco_git/script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="143" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{932B8B02-9110-4A78-97CD-3791BC1D5F25}"/>
+  <xr:revisionPtr revIDLastSave="153" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95AFD35-4997-47B1-80CF-B272FEFB4D00}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1830" windowWidth="26595" windowHeight="13770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="simulation_queue" sheetId="1" r:id="rId1"/>
     <sheet name="completed_queue" sheetId="2" r:id="rId2"/>
     <sheet name="models" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="0" fullCalcOnLoad="true"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="484" uniqueCount="112">
   <si>
     <t>SF</t>
   </si>
@@ -419,15 +419,12 @@
     <t>test1</t>
     <phoneticPr fontId="18" type="noConversion"/>
   </si>
-  <si>
-    <t>2D_gait_AFO_pc_50kg.osim</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -637,19 +634,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79995117038483843"/>
+        <fgColor theme="4" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59996337778862885"/>
+        <fgColor theme="4" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
+        <fgColor theme="4" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -660,19 +657,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79995117038483843"/>
+        <fgColor theme="5" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59996337778862885"/>
+        <fgColor theme="5" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
+        <fgColor theme="5" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -683,19 +680,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79995117038483843"/>
+        <fgColor theme="6" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59996337778862885"/>
+        <fgColor theme="6" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
+        <fgColor theme="6" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -706,19 +703,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79995117038483843"/>
+        <fgColor theme="7" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59996337778862885"/>
+        <fgColor theme="7" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
+        <fgColor theme="7" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -729,19 +726,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79995117038483843"/>
+        <fgColor theme="8" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59996337778862885"/>
+        <fgColor theme="8" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
+        <fgColor theme="8" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -752,24 +749,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79995117038483843"/>
+        <fgColor theme="9" tint="0.79995117038484"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59996337778862885"/>
+        <fgColor theme="9" tint="0.59996337778863"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
+        <fgColor theme="9" tint="0.39997558519242"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="10">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -791,7 +788,7 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.49995422223578601"/>
+        <color theme="4" tint="0.49995422223579"/>
       </bottom>
       <diagonal/>
     </border>
@@ -800,7 +797,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
+        <color theme="4" tint="0.39997558519242"/>
       </bottom>
       <diagonal/>
     </border>
@@ -884,191 +881,193 @@
       </bottom>
       <diagonal/>
     </border>
+    <border/>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="false" applyFont="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment vertical="center" wrapText="true"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyAlignment="true">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="1"/>
-    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="1"/>
-    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="true"/>
+    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="true"/>
+    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="true"/>
+    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="true"/>
+    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="true"/>
+    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="true"/>
+    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="true"/>
+    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="true"/>
+    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="true"/>
+    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="true"/>
+    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="true"/>
+    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="true"/>
+    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="true"/>
+    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="true"/>
+    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="true"/>
+    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="true"/>
+    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="true"/>
+    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="true"/>
+    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="true"/>
+    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="true"/>
+    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="true"/>
+    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="true"/>
+    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="true"/>
+    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="true"/>
+    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="true"/>
+    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="true"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1085,7 +1084,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1236,7 +1235,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1260,9 +1259,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1286,7 +1285,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1321,7 +1320,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1339,7 +1338,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill rotWithShape="true">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1364,7 +1363,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="5400000" scaled="false"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1380,468 +1379,674 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U18"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:U17"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.75" customWidth="1"/>
-    <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="24.75" customWidth="1"/>
-    <col min="4" max="4" width="4" customWidth="1"/>
-    <col min="5" max="5" width="13.5" customWidth="1"/>
-    <col min="6" max="6" width="6.875" customWidth="1"/>
-    <col min="7" max="7" width="4.125" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="3.875" customWidth="1"/>
-    <col min="10" max="10" width="7.5" customWidth="1"/>
-    <col min="11" max="11" width="14.375" customWidth="1"/>
-    <col min="12" max="12" width="9.25" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="4.625" customWidth="1"/>
-    <col min="15" max="15" width="10.625" customWidth="1"/>
-    <col min="16" max="16" width="14.125" customWidth="1"/>
-    <col min="17" max="17" width="15.75" customWidth="1"/>
-    <col min="18" max="18" width="14.875" customWidth="1"/>
-    <col min="19" max="19" width="10.625" customWidth="1"/>
-    <col min="20" max="20" width="12.875" customWidth="1"/>
-    <col min="21" max="21" width="9.5" customWidth="1"/>
+    <col min="1" max="1" width="25.75" customWidth="true"/>
+    <col min="2" max="2" width="10" customWidth="true"/>
+    <col min="3" max="3" width="22.75" customWidth="true"/>
+    <col min="4" max="4" width="4" customWidth="true"/>
+    <col min="5" max="5" width="13.5" customWidth="true"/>
+    <col min="6" max="6" width="6.875" customWidth="true"/>
+    <col min="7" max="7" width="4.125" customWidth="true"/>
+    <col min="8" max="8" width="4" customWidth="true"/>
+    <col min="9" max="9" width="3.875" customWidth="true"/>
+    <col min="10" max="10" width="7.5" customWidth="true"/>
+    <col min="11" max="11" width="14.375" customWidth="true"/>
+    <col min="12" max="12" width="9.25" customWidth="true"/>
+    <col min="13" max="13" width="11" customWidth="true"/>
+    <col min="14" max="14" width="4.625" customWidth="true"/>
+    <col min="15" max="15" width="10.625" customWidth="true"/>
+    <col min="16" max="16" width="14.125" customWidth="true"/>
+    <col min="17" max="17" width="15.75" customWidth="true"/>
+    <col min="18" max="18" width="14.875" customWidth="true"/>
+    <col min="19" max="19" width="10.625" customWidth="true"/>
+    <col min="20" max="20" width="12.875" customWidth="true"/>
+    <col min="21" max="21" width="9.5" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="2">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="K2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="0"/>
+      <c r="P2" s="0"/>
+      <c r="Q2" s="0"/>
+      <c r="R2" s="0"/>
+      <c r="S2" s="0"/>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="K3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="0"/>
+      <c r="P3" s="0"/>
+      <c r="Q3" s="0"/>
+      <c r="R3" s="0"/>
+      <c r="S3" s="0"/>
+      <c r="T3" s="0"/>
+      <c r="U3" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="2">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+        <v>0.029999999999999999</v>
+      </c>
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="0"/>
+      <c r="P4" s="0"/>
+      <c r="Q4" s="0"/>
+      <c r="R4" s="0"/>
+      <c r="S4" s="0"/>
+      <c r="T4" s="0"/>
+      <c r="U4" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0"/>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0"/>
+      <c r="T5" s="0"/>
+      <c r="U5" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="0"/>
+      <c r="P6" s="0"/>
+      <c r="Q6" s="0"/>
+      <c r="R6" s="0"/>
+      <c r="S6" s="0"/>
+      <c r="T6" s="0"/>
+      <c r="U6" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:21" ht="165" x14ac:dyDescent="0.3">
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+      <c r="S7" s="0"/>
+      <c r="T7" s="0"/>
+      <c r="U7" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" ht="165" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="2"/>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+      <c r="S8" s="0"/>
+      <c r="T8" s="0"/>
+      <c r="U8" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B9" s="2"/>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="C9" s="0"/>
+      <c r="D9" s="0"/>
+      <c r="E9" s="0"/>
+      <c r="F9" s="0"/>
+      <c r="G9" s="0"/>
+      <c r="H9" s="0"/>
+      <c r="I9" s="0"/>
+      <c r="J9" s="0"/>
+      <c r="K9" s="0"/>
+      <c r="L9" s="0"/>
+      <c r="M9" s="0"/>
+      <c r="N9" s="0"/>
+      <c r="O9" s="0"/>
+      <c r="P9" s="0"/>
+      <c r="Q9" s="0"/>
+      <c r="R9" s="0"/>
+      <c r="S9" s="0"/>
+      <c r="T9" s="0"/>
+      <c r="U9" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="L10" t="s">
+      <c r="L10" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="M10" t="s">
+      <c r="M10" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="N10" t="s">
+      <c r="N10" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="O10" t="s">
+      <c r="O10" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="P10" t="s">
+      <c r="P10" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" t="s">
+      <c r="Q10" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="S10" t="s">
+      <c r="S10" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="T10" t="s">
+      <c r="T10" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="U10" t="s">
+      <c r="U10" s="0" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+      <c r="A11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="0">
         <v>260515</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>100</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>3</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K11" t="s">
+      <c r="F11" s="0"/>
+      <c r="G11" s="0"/>
+      <c r="H11" s="0"/>
+      <c r="I11" s="0"/>
+      <c r="J11" s="0"/>
+      <c r="K11" s="0" t="s">
         <v>99</v>
       </c>
-      <c r="O11">
-        <v>1</v>
-      </c>
-      <c r="P11">
-        <v>1.0999999999999999E-2</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0">
+        <v>0.010999999999999999</v>
+      </c>
+      <c r="Q11" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U11">
+      <c r="T11" s="0"/>
+      <c r="U11" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+      <c r="A12" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="0">
         <v>260515</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>102</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="0">
         <v>3</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K12" t="s">
+      <c r="F12" s="0"/>
+      <c r="G12" s="0"/>
+      <c r="H12" s="0"/>
+      <c r="I12" s="0"/>
+      <c r="J12" s="0"/>
+      <c r="K12" s="0" t="s">
         <v>101</v>
       </c>
-      <c r="O12">
-        <v>1</v>
-      </c>
-      <c r="P12">
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0">
+        <v>1</v>
+      </c>
+      <c r="P12" s="0">
         <v>0.70099999999999996</v>
       </c>
-      <c r="Q12" t="s">
+      <c r="Q12" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S12" t="s">
+      <c r="S12" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U12">
+      <c r="T12" s="0"/>
+      <c r="U12" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+      <c r="A13" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="0">
         <v>260515</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>104</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K13" t="s">
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="K13" s="0" t="s">
         <v>103</v>
       </c>
-      <c r="O13">
-        <v>1</v>
-      </c>
-      <c r="P13">
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="0">
+        <v>1</v>
+      </c>
+      <c r="P13" s="0">
         <v>0.10100000000000001</v>
       </c>
-      <c r="Q13" t="s">
+      <c r="Q13" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R13" t="s">
+      <c r="R13" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S13" t="s">
+      <c r="S13" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U13">
+      <c r="T13" s="0"/>
+      <c r="U13" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+      <c r="A14" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="0">
         <v>260515</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="0">
         <v>3</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K14" t="s">
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="K14" s="0" t="s">
         <v>105</v>
       </c>
-      <c r="O14">
-        <v>1</v>
-      </c>
-      <c r="P14">
-        <v>5.0999999999999997E-2</v>
-      </c>
-      <c r="Q14" t="s">
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="0">
+        <v>1</v>
+      </c>
+      <c r="P14" s="0">
+        <v>0.050999999999999997</v>
+      </c>
+      <c r="Q14" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R14" t="s">
+      <c r="R14" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S14" t="s">
+      <c r="S14" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U14">
+      <c r="T14" s="0"/>
+      <c r="U14" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="0">
         <v>260515</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="0" t="s">
         <v>106</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="0">
         <v>3</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K15" t="s">
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0" t="s">
         <v>107</v>
       </c>
-      <c r="O15">
-        <v>1</v>
-      </c>
-      <c r="P15">
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0">
+        <v>1</v>
+      </c>
+      <c r="P15" s="0">
         <v>1.0049999999999999</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="Q15" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R15" t="s">
+      <c r="R15" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S15" t="s">
+      <c r="S15" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U15">
+      <c r="T15" s="0"/>
+      <c r="U15" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+      <c r="A16" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="0">
         <v>260515</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="0" t="s">
         <v>109</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="0">
         <v>3</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K16" t="s">
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0" t="s">
         <v>108</v>
       </c>
-      <c r="O16">
-        <v>1</v>
-      </c>
-      <c r="P16">
+      <c r="L16" s="0"/>
+      <c r="M16" s="0"/>
+      <c r="N16" s="0"/>
+      <c r="O16" s="0">
+        <v>1</v>
+      </c>
+      <c r="P16" s="0">
         <v>2.0049999999999999</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="Q16" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U16">
+      <c r="T16" s="0"/>
+      <c r="U16" s="0">
         <v>-1</v>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+      <c r="A17" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="B17">
-        <v>260605</v>
-      </c>
-      <c r="C17" t="s">
-        <v>110</v>
-      </c>
-      <c r="D17">
+      <c r="B17" s="0">
+        <v>260615</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="D17" s="0">
         <v>3</v>
       </c>
-      <c r="E17" t="s">
-        <v>73</v>
-      </c>
-      <c r="K17" t="s">
+      <c r="E17" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="F17" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="G17" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="H17" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="I17" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J17" s="0">
+        <v>1</v>
+      </c>
+      <c r="K17" s="0" t="s">
         <v>111</v>
       </c>
-      <c r="O17">
-        <v>1</v>
-      </c>
-      <c r="P17">
-        <v>1E-3</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="L17" s="0"/>
+      <c r="M17" s="0"/>
+      <c r="N17" s="0"/>
+      <c r="O17" s="0">
+        <v>1</v>
+      </c>
+      <c r="P17" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q17" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R17" t="s">
+      <c r="R17" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S17" t="s">
+      <c r="S17" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
-        <v>111</v>
-      </c>
-      <c r="B18">
-        <v>260610</v>
-      </c>
-      <c r="C18" t="s">
-        <v>112</v>
-      </c>
-      <c r="D18">
-        <v>3</v>
-      </c>
-      <c r="E18" t="s">
-        <v>73</v>
-      </c>
-      <c r="K18" t="s">
-        <v>111</v>
-      </c>
-      <c r="O18">
-        <v>1</v>
-      </c>
-      <c r="P18">
-        <v>1E-3</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>74</v>
-      </c>
-      <c r="R18" t="s">
-        <v>28</v>
-      </c>
-      <c r="S18" t="s">
-        <v>75</v>
-      </c>
-      <c r="U18">
-        <v>0</v>
+      <c r="T17" s="0"/>
+      <c r="U17" s="0">
+        <v>-1</v>
       </c>
     </row>
   </sheetData>
@@ -1852,686 +2057,944 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
   <dimension ref="A1:U22"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.375" customWidth="1"/>
-    <col min="2" max="2" width="7.25" customWidth="1"/>
-    <col min="3" max="3" width="24.75" customWidth="1"/>
-    <col min="4" max="4" width="4" customWidth="1"/>
-    <col min="5" max="5" width="13.5" customWidth="1"/>
-    <col min="6" max="6" width="6.875" customWidth="1"/>
-    <col min="7" max="7" width="4.125" customWidth="1"/>
-    <col min="8" max="8" width="4" customWidth="1"/>
-    <col min="9" max="9" width="3.875" customWidth="1"/>
-    <col min="10" max="10" width="7.5" customWidth="1"/>
-    <col min="11" max="11" width="11.375" customWidth="1"/>
-    <col min="12" max="12" width="9.25" customWidth="1"/>
-    <col min="13" max="13" width="11" customWidth="1"/>
-    <col min="14" max="14" width="4.625" customWidth="1"/>
-    <col min="15" max="15" width="10.625" customWidth="1"/>
-    <col min="16" max="16" width="14.125" customWidth="1"/>
-    <col min="17" max="17" width="15.75" customWidth="1"/>
-    <col min="18" max="18" width="14.875" customWidth="1"/>
-    <col min="19" max="19" width="10.625" customWidth="1"/>
-    <col min="20" max="20" width="12.875" customWidth="1"/>
-    <col min="21" max="21" width="9.5" customWidth="1"/>
+    <col min="1" max="1" width="10.375" customWidth="true"/>
+    <col min="2" max="2" width="7.25" customWidth="true"/>
+    <col min="3" max="3" width="24.75" customWidth="true"/>
+    <col min="4" max="4" width="4" customWidth="true"/>
+    <col min="5" max="5" width="13.5" customWidth="true"/>
+    <col min="6" max="6" width="6.875" customWidth="true"/>
+    <col min="7" max="7" width="4.125" customWidth="true"/>
+    <col min="8" max="8" width="4" customWidth="true"/>
+    <col min="9" max="9" width="3.875" customWidth="true"/>
+    <col min="10" max="10" width="7.5" customWidth="true"/>
+    <col min="11" max="11" width="11.375" customWidth="true"/>
+    <col min="12" max="12" width="9.25" customWidth="true"/>
+    <col min="13" max="13" width="11" customWidth="true"/>
+    <col min="14" max="14" width="4.625" customWidth="true"/>
+    <col min="15" max="15" width="10.625" customWidth="true"/>
+    <col min="16" max="16" width="14.125" customWidth="true"/>
+    <col min="17" max="17" width="15.75" customWidth="true"/>
+    <col min="18" max="18" width="14.875" customWidth="true"/>
+    <col min="19" max="19" width="10.625" customWidth="true"/>
+    <col min="20" max="20" width="12.875" customWidth="true"/>
+    <col min="21" max="21" width="9.5" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2">
+      <c r="B1" s="0">
+        <v>1</v>
+      </c>
+      <c r="C1" s="0"/>
+      <c r="D1" s="0"/>
+      <c r="E1" s="0"/>
+      <c r="F1" s="0"/>
+      <c r="G1" s="0"/>
+      <c r="H1" s="0"/>
+      <c r="I1" s="0"/>
+      <c r="J1" s="0"/>
+      <c r="K1" s="0"/>
+      <c r="L1" s="0"/>
+      <c r="M1" s="0"/>
+      <c r="N1" s="0"/>
+      <c r="O1" s="0"/>
+      <c r="P1" s="0"/>
+      <c r="Q1" s="0"/>
+      <c r="R1" s="0"/>
+      <c r="S1" s="0"/>
+      <c r="T1" s="0"/>
+      <c r="U1" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+      <c r="A2" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="C2" s="0"/>
+      <c r="D2" s="0"/>
+      <c r="E2" s="0"/>
+      <c r="F2" s="0"/>
+      <c r="G2" s="0"/>
+      <c r="H2" s="0"/>
+      <c r="I2" s="0"/>
+      <c r="J2" s="0"/>
+      <c r="K2" s="0"/>
+      <c r="L2" s="0"/>
+      <c r="M2" s="0"/>
+      <c r="N2" s="0"/>
+      <c r="O2" s="0"/>
+      <c r="P2" s="0"/>
+      <c r="Q2" s="0"/>
+      <c r="R2" s="0"/>
+      <c r="S2" s="0"/>
+      <c r="T2" s="0"/>
+      <c r="U2" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+      <c r="A3" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="C3" s="0"/>
+      <c r="D3" s="0"/>
+      <c r="E3" s="0"/>
+      <c r="F3" s="0"/>
+      <c r="G3" s="0"/>
+      <c r="H3" s="0"/>
+      <c r="I3" s="0"/>
+      <c r="J3" s="0"/>
+      <c r="K3" s="0"/>
+      <c r="L3" s="0"/>
+      <c r="M3" s="0"/>
+      <c r="N3" s="0"/>
+      <c r="O3" s="0"/>
+      <c r="P3" s="0"/>
+      <c r="Q3" s="0"/>
+      <c r="R3" s="0"/>
+      <c r="S3" s="0"/>
+      <c r="T3" s="0"/>
+      <c r="U3" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+      <c r="A4" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="C4" s="0"/>
+      <c r="D4" s="0"/>
+      <c r="E4" s="0"/>
+      <c r="F4" s="0"/>
+      <c r="G4" s="0"/>
+      <c r="H4" s="0"/>
+      <c r="I4" s="0"/>
+      <c r="J4" s="0"/>
+      <c r="K4" s="0"/>
+      <c r="L4" s="0"/>
+      <c r="M4" s="0"/>
+      <c r="N4" s="0"/>
+      <c r="O4" s="0"/>
+      <c r="P4" s="0"/>
+      <c r="Q4" s="0"/>
+      <c r="R4" s="0"/>
+      <c r="S4" s="0"/>
+      <c r="T4" s="0"/>
+      <c r="U4" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+      <c r="A5" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="C5" s="0"/>
+      <c r="D5" s="0"/>
+      <c r="E5" s="0"/>
+      <c r="F5" s="0"/>
+      <c r="G5" s="0"/>
+      <c r="H5" s="0"/>
+      <c r="I5" s="0"/>
+      <c r="J5" s="0"/>
+      <c r="K5" s="0"/>
+      <c r="L5" s="0"/>
+      <c r="M5" s="0"/>
+      <c r="N5" s="0"/>
+      <c r="O5" s="0"/>
+      <c r="P5" s="0"/>
+      <c r="Q5" s="0"/>
+      <c r="R5" s="0"/>
+      <c r="S5" s="0"/>
+      <c r="T5" s="0"/>
+      <c r="U5" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+      <c r="A6" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="0">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="C6" s="0"/>
+      <c r="D6" s="0"/>
+      <c r="E6" s="0"/>
+      <c r="F6" s="0"/>
+      <c r="G6" s="0"/>
+      <c r="H6" s="0"/>
+      <c r="I6" s="0"/>
+      <c r="J6" s="0"/>
+      <c r="K6" s="0"/>
+      <c r="L6" s="0"/>
+      <c r="M6" s="0"/>
+      <c r="N6" s="0"/>
+      <c r="O6" s="0"/>
+      <c r="P6" s="0"/>
+      <c r="Q6" s="0"/>
+      <c r="R6" s="0"/>
+      <c r="S6" s="0"/>
+      <c r="T6" s="0"/>
+      <c r="U6" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+      <c r="A7" s="0" t="s">
         <v>76</v>
       </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="B7" s="0">
+        <v>1</v>
+      </c>
+      <c r="C7" s="0"/>
+      <c r="D7" s="0"/>
+      <c r="E7" s="0"/>
+      <c r="F7" s="0"/>
+      <c r="G7" s="0"/>
+      <c r="H7" s="0"/>
+      <c r="I7" s="0"/>
+      <c r="J7" s="0"/>
+      <c r="K7" s="0"/>
+      <c r="L7" s="0"/>
+      <c r="M7" s="0"/>
+      <c r="N7" s="0"/>
+      <c r="O7" s="0"/>
+      <c r="P7" s="0"/>
+      <c r="Q7" s="0"/>
+      <c r="R7" s="0"/>
+      <c r="S7" s="0"/>
+      <c r="T7" s="0"/>
+      <c r="U7" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+      <c r="A8" s="0" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="B8" s="0"/>
+      <c r="C8" s="0"/>
+      <c r="D8" s="0"/>
+      <c r="E8" s="0"/>
+      <c r="F8" s="0"/>
+      <c r="G8" s="0"/>
+      <c r="H8" s="0"/>
+      <c r="I8" s="0"/>
+      <c r="J8" s="0"/>
+      <c r="K8" s="0"/>
+      <c r="L8" s="0"/>
+      <c r="M8" s="0"/>
+      <c r="N8" s="0"/>
+      <c r="O8" s="0"/>
+      <c r="P8" s="0"/>
+      <c r="Q8" s="0"/>
+      <c r="R8" s="0"/>
+      <c r="S8" s="0"/>
+      <c r="T8" s="0"/>
+      <c r="U8" s="0"/>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+      <c r="A9" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="L9" t="s">
+      <c r="L9" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="M9" t="s">
+      <c r="M9" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="N9" t="s">
+      <c r="N9" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="O9" t="s">
+      <c r="O9" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="P9" t="s">
+      <c r="P9" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="Q9" t="s">
+      <c r="Q9" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="R9" t="s">
+      <c r="R9" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="S9" t="s">
+      <c r="S9" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="T9" t="s">
+      <c r="T9" s="0" t="s">
         <v>24</v>
       </c>
-      <c r="U9" t="s">
+      <c r="U9" s="0" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+      <c r="A10" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="0">
         <v>260501</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="0" t="s">
         <v>62</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="0">
         <v>3</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F10">
-        <v>0.2</v>
-      </c>
-      <c r="G10">
-        <v>0.3</v>
-      </c>
-      <c r="H10">
+      <c r="F10" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G10" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H10" s="0">
         <v>0</v>
       </c>
-      <c r="I10">
-        <v>0.1</v>
-      </c>
-      <c r="J10">
-        <v>1</v>
-      </c>
-      <c r="K10" t="s">
+      <c r="I10" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J10" s="0">
+        <v>1</v>
+      </c>
+      <c r="K10" s="0" t="s">
         <v>77</v>
       </c>
-      <c r="O10">
-        <v>1</v>
-      </c>
-      <c r="P10">
-        <v>1E-4</v>
-      </c>
-      <c r="Q10" t="s">
+      <c r="L10" s="0"/>
+      <c r="M10" s="0"/>
+      <c r="N10" s="0"/>
+      <c r="O10" s="0">
+        <v>1</v>
+      </c>
+      <c r="P10" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q10" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R10" t="s">
+      <c r="R10" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S10" t="s">
+      <c r="S10" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="T10" s="0"/>
+      <c r="U10" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+      <c r="A11" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="0">
         <v>260501</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="0">
         <v>3</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F11">
-        <v>0.2</v>
-      </c>
-      <c r="G11">
-        <v>0.3</v>
-      </c>
-      <c r="H11">
+      <c r="F11" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G11" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H11" s="0">
         <v>0</v>
       </c>
-      <c r="I11">
-        <v>0.1</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="I11" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J11" s="0">
+        <v>1</v>
+      </c>
+      <c r="K11" s="0" t="s">
         <v>81</v>
       </c>
-      <c r="O11">
-        <v>1</v>
-      </c>
-      <c r="P11">
-        <v>1E-4</v>
-      </c>
-      <c r="Q11" t="s">
+      <c r="L11" s="0"/>
+      <c r="M11" s="0"/>
+      <c r="N11" s="0"/>
+      <c r="O11" s="0">
+        <v>1</v>
+      </c>
+      <c r="P11" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q11" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R11" t="s">
+      <c r="R11" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S11" t="s">
+      <c r="S11" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="T11" s="0"/>
+      <c r="U11" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+      <c r="A12" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="0">
         <v>260501</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="0" t="s">
         <v>64</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="0">
         <v>3</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="0" t="s">
         <v>78</v>
       </c>
-      <c r="F12">
-        <v>0.2</v>
-      </c>
-      <c r="G12">
-        <v>0.3</v>
-      </c>
-      <c r="H12">
+      <c r="F12" s="0">
+        <v>0.20000000000000001</v>
+      </c>
+      <c r="G12" s="0">
+        <v>0.29999999999999999</v>
+      </c>
+      <c r="H12" s="0">
         <v>0</v>
       </c>
-      <c r="I12">
-        <v>0.1</v>
-      </c>
-      <c r="J12">
-        <v>1</v>
-      </c>
-      <c r="K12" t="s">
+      <c r="I12" s="0">
+        <v>0.10000000000000001</v>
+      </c>
+      <c r="J12" s="0">
+        <v>1</v>
+      </c>
+      <c r="K12" s="0" t="s">
         <v>82</v>
       </c>
-      <c r="O12">
-        <v>1</v>
-      </c>
-      <c r="P12">
-        <v>1E-4</v>
-      </c>
-      <c r="Q12" t="s">
+      <c r="L12" s="0"/>
+      <c r="M12" s="0"/>
+      <c r="N12" s="0"/>
+      <c r="O12" s="0">
+        <v>1</v>
+      </c>
+      <c r="P12" s="0">
+        <v>0.0001</v>
+      </c>
+      <c r="Q12" s="0" t="s">
         <v>79</v>
       </c>
-      <c r="R12" t="s">
+      <c r="R12" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="S12" t="s">
+      <c r="S12" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="T12" s="0"/>
+      <c r="U12" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+      <c r="A13" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="B13">
+      <c r="B13" s="0">
         <v>260513</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="0" t="s">
         <v>65</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="0">
         <v>3</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K13" t="s">
+      <c r="F13" s="0"/>
+      <c r="G13" s="0"/>
+      <c r="H13" s="0"/>
+      <c r="I13" s="0"/>
+      <c r="J13" s="0"/>
+      <c r="K13" s="0" t="s">
         <v>83</v>
       </c>
-      <c r="S13" t="s">
+      <c r="L13" s="0"/>
+      <c r="M13" s="0"/>
+      <c r="N13" s="0"/>
+      <c r="O13" s="0"/>
+      <c r="P13" s="0"/>
+      <c r="Q13" s="0"/>
+      <c r="R13" s="0"/>
+      <c r="S13" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="T13" s="0"/>
+      <c r="U13" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+      <c r="A14" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="0">
         <v>260513</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="0" t="s">
         <v>86</v>
       </c>
-      <c r="D14">
+      <c r="D14" s="0">
         <v>3</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K14" t="s">
+      <c r="F14" s="0"/>
+      <c r="G14" s="0"/>
+      <c r="H14" s="0"/>
+      <c r="I14" s="0"/>
+      <c r="J14" s="0"/>
+      <c r="K14" s="0" t="s">
         <v>85</v>
       </c>
-      <c r="S14" t="s">
+      <c r="L14" s="0"/>
+      <c r="M14" s="0"/>
+      <c r="N14" s="0"/>
+      <c r="O14" s="0"/>
+      <c r="P14" s="0"/>
+      <c r="Q14" s="0"/>
+      <c r="R14" s="0"/>
+      <c r="S14" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="T14" s="0"/>
+      <c r="U14" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+      <c r="A15" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="0">
         <v>260513</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="0">
         <v>3</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K15" t="s">
+      <c r="F15" s="0"/>
+      <c r="G15" s="0"/>
+      <c r="H15" s="0"/>
+      <c r="I15" s="0"/>
+      <c r="J15" s="0"/>
+      <c r="K15" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="S15" t="s">
+      <c r="L15" s="0"/>
+      <c r="M15" s="0"/>
+      <c r="N15" s="0"/>
+      <c r="O15" s="0"/>
+      <c r="P15" s="0"/>
+      <c r="Q15" s="0"/>
+      <c r="R15" s="0"/>
+      <c r="S15" s="0" t="s">
         <v>84</v>
       </c>
-      <c r="U15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="T15" s="0"/>
+      <c r="U15" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+      <c r="A16" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="B16">
+      <c r="B16" s="0">
         <v>260419</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="D16">
+      <c r="D16" s="0">
         <v>3</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K16" t="s">
+      <c r="F16" s="0"/>
+      <c r="G16" s="0"/>
+      <c r="H16" s="0"/>
+      <c r="I16" s="0"/>
+      <c r="J16" s="0"/>
+      <c r="K16" s="0" t="s">
         <v>89</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="0">
         <v>0.01</v>
       </c>
-      <c r="M16">
+      <c r="M16" s="0">
         <v>0</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N16" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O16">
-        <v>1</v>
-      </c>
-      <c r="P16">
-        <v>1E-3</v>
-      </c>
-      <c r="Q16" t="s">
+      <c r="O16" s="0">
+        <v>1</v>
+      </c>
+      <c r="P16" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q16" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R16" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S16" t="s">
+      <c r="S16" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="T16" s="0"/>
+      <c r="U16" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+      <c r="A17" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="B17">
+      <c r="B17" s="0">
         <v>260419</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="D17">
+      <c r="D17" s="0">
         <v>3</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K17" t="s">
+      <c r="F17" s="0"/>
+      <c r="G17" s="0"/>
+      <c r="H17" s="0"/>
+      <c r="I17" s="0"/>
+      <c r="J17" s="0"/>
+      <c r="K17" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="0">
         <v>0.01</v>
       </c>
-      <c r="M17">
+      <c r="M17" s="0">
         <v>0</v>
       </c>
-      <c r="N17" t="s">
+      <c r="N17" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O17">
-        <v>1</v>
-      </c>
-      <c r="P17">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="Q17" t="s">
+      <c r="O17" s="0">
+        <v>1</v>
+      </c>
+      <c r="P17" s="0">
+        <v>0.0050000000000000001</v>
+      </c>
+      <c r="Q17" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R17" t="s">
+      <c r="R17" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S17" t="s">
+      <c r="S17" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="T17" s="0"/>
+      <c r="U17" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+      <c r="A18" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="B18">
+      <c r="B18" s="0">
         <v>260419</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="0" t="s">
         <v>110</v>
       </c>
-      <c r="D18">
+      <c r="D18" s="0">
         <v>3</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="0" t="s">
         <v>90</v>
       </c>
-      <c r="K18" t="s">
+      <c r="F18" s="0"/>
+      <c r="G18" s="0"/>
+      <c r="H18" s="0"/>
+      <c r="I18" s="0"/>
+      <c r="J18" s="0"/>
+      <c r="K18" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="0">
         <v>0.01</v>
       </c>
-      <c r="M18">
+      <c r="M18" s="0">
         <v>0</v>
       </c>
-      <c r="N18" t="s">
+      <c r="N18" s="0" t="s">
         <v>91</v>
       </c>
-      <c r="O18">
-        <v>1</v>
-      </c>
-      <c r="P18">
+      <c r="O18" s="0">
+        <v>1</v>
+      </c>
+      <c r="P18" s="0">
         <v>0.01</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="Q18" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R18" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S18" t="s">
+      <c r="S18" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="T18" s="0"/>
+      <c r="U18" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+      <c r="A19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B19">
+      <c r="B19" s="0">
         <v>260416</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D19">
+      <c r="D19" s="0">
         <v>3</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K19" t="s">
+      <c r="F19" s="0"/>
+      <c r="G19" s="0"/>
+      <c r="H19" s="0"/>
+      <c r="I19" s="0"/>
+      <c r="J19" s="0"/>
+      <c r="K19" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="O19">
-        <v>1</v>
-      </c>
-      <c r="P19">
-        <v>1E-3</v>
-      </c>
-      <c r="Q19" t="s">
+      <c r="L19" s="0"/>
+      <c r="M19" s="0"/>
+      <c r="N19" s="0"/>
+      <c r="O19" s="0">
+        <v>1</v>
+      </c>
+      <c r="P19" s="0">
+        <v>0.001</v>
+      </c>
+      <c r="Q19" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R19" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S19" t="s">
+      <c r="S19" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="T19" s="0"/>
+      <c r="U19" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+      <c r="A20" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="B20">
+      <c r="B20" s="0">
         <v>260416</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D20">
+      <c r="D20" s="0">
         <v>3</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K20" t="s">
+      <c r="F20" s="0"/>
+      <c r="G20" s="0"/>
+      <c r="H20" s="0"/>
+      <c r="I20" s="0"/>
+      <c r="J20" s="0"/>
+      <c r="K20" s="0" t="s">
         <v>96</v>
       </c>
-      <c r="O20">
-        <v>1</v>
-      </c>
-      <c r="P20">
-        <v>5.0000000000000001E-3</v>
-      </c>
-      <c r="Q20" t="s">
+      <c r="L20" s="0"/>
+      <c r="M20" s="0"/>
+      <c r="N20" s="0"/>
+      <c r="O20" s="0">
+        <v>1</v>
+      </c>
+      <c r="P20" s="0">
+        <v>0.0050000000000000001</v>
+      </c>
+      <c r="Q20" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R20" t="s">
+      <c r="R20" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S20" t="s">
+      <c r="S20" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="T20" s="0"/>
+      <c r="U20" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+      <c r="A21" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="B21">
+      <c r="B21" s="0">
         <v>260416</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D21">
+      <c r="D21" s="0">
         <v>3</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K21" t="s">
+      <c r="F21" s="0"/>
+      <c r="G21" s="0"/>
+      <c r="H21" s="0"/>
+      <c r="I21" s="0"/>
+      <c r="J21" s="0"/>
+      <c r="K21" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="O21">
-        <v>1</v>
-      </c>
-      <c r="P21">
+      <c r="L21" s="0"/>
+      <c r="M21" s="0"/>
+      <c r="N21" s="0"/>
+      <c r="O21" s="0">
+        <v>1</v>
+      </c>
+      <c r="P21" s="0">
         <v>0.01</v>
       </c>
-      <c r="Q21" t="s">
+      <c r="Q21" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R21" t="s">
+      <c r="R21" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S21" t="s">
+      <c r="S21" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="T21" s="0"/>
+      <c r="U21" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+      <c r="A22" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="B22">
+      <c r="B22" s="0">
         <v>260416</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="0" t="s">
         <v>95</v>
       </c>
-      <c r="D22">
+      <c r="D22" s="0">
         <v>3</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="0" t="s">
         <v>73</v>
       </c>
-      <c r="K22" t="s">
+      <c r="F22" s="0"/>
+      <c r="G22" s="0"/>
+      <c r="H22" s="0"/>
+      <c r="I22" s="0"/>
+      <c r="J22" s="0"/>
+      <c r="K22" s="0" t="s">
         <v>98</v>
       </c>
-      <c r="O22">
-        <v>1</v>
-      </c>
-      <c r="P22">
-        <v>0.03</v>
-      </c>
-      <c r="Q22" t="s">
+      <c r="L22" s="0"/>
+      <c r="M22" s="0"/>
+      <c r="N22" s="0"/>
+      <c r="O22" s="0">
+        <v>1</v>
+      </c>
+      <c r="P22" s="0">
+        <v>0.029999999999999999</v>
+      </c>
+      <c r="Q22" s="0" t="s">
         <v>74</v>
       </c>
-      <c r="R22" t="s">
+      <c r="R22" s="0" t="s">
         <v>28</v>
       </c>
-      <c r="S22" t="s">
+      <c r="S22" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="U22">
+      <c r="T22" s="0"/>
+      <c r="U22" s="0">
         <v>1</v>
       </c>
     </row>
@@ -2543,20 +3006,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.375" customWidth="1"/>
-    <col min="2" max="2" width="24.75" customWidth="1"/>
-    <col min="3" max="3" width="7.25" customWidth="1"/>
-    <col min="4" max="4" width="5.75" customWidth="1"/>
-    <col min="5" max="5" width="6.25" customWidth="1"/>
-    <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="9.375" customWidth="1"/>
+    <col min="1" max="1" width="27.375" customWidth="true"/>
+    <col min="2" max="2" width="24.75" customWidth="true"/>
+    <col min="3" max="3" width="7.25" customWidth="true"/>
+    <col min="4" max="4" width="5.75" customWidth="true"/>
+    <col min="5" max="5" width="6.25" customWidth="true"/>
+    <col min="6" max="6" width="4" customWidth="true"/>
+    <col min="7" max="7" width="9.375" customWidth="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -2564,7 +3027,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -2572,7 +3035,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -2580,12 +3043,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -2608,7 +3071,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -2625,7 +3088,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -2642,7 +3105,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -2659,7 +3122,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -2676,7 +3139,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -2693,7 +3156,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -2710,7 +3173,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -2727,7 +3190,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -2744,7 +3207,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -2761,7 +3224,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -2778,7 +3241,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -2795,7 +3258,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -2812,7 +3275,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -2829,7 +3292,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -2846,7 +3309,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -2863,7 +3326,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -2880,7 +3343,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -2897,7 +3360,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -2914,7 +3377,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -2931,7 +3394,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -2948,7 +3411,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>68</v>
       </c>
@@ -2965,7 +3428,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -2982,7 +3445,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -2999,7 +3462,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>71</v>
       </c>
@@ -3016,7 +3479,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>72</v>
       </c>

</xml_diff>

<commit_message>
update minor scripts difference
</commit_message>
<xml_diff>
--- a/script/simulation_queue_example.xlsx
+++ b/script/simulation_queue_example.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5f03addda2663411/SRBL/WearableOptimizedControl/Optimizer/Moco_git/script/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="153" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F95AFD35-4997-47B1-80CF-B272FEFB4D00}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="8_{985CFB64-8444-49E3-9649-B21738068EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{504CF446-CE45-4A62-A37C-FC62B2239A02}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="simulation_queue" sheetId="1" r:id="rId1"/>
     <sheet name="completed_queue" sheetId="2" r:id="rId2"/>
     <sheet name="models" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0" fullCalcOnLoad="true"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="484" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="112">
   <si>
     <t>SF</t>
   </si>
@@ -423,8 +423,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <fonts count="19">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -634,19 +634,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79995117038484"/>
+        <fgColor theme="4" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59996337778863"/>
+        <fgColor theme="4" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519242"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -657,19 +657,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79995117038484"/>
+        <fgColor theme="5" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59996337778863"/>
+        <fgColor theme="5" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519242"/>
+        <fgColor theme="5" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -680,19 +680,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79995117038484"/>
+        <fgColor theme="6" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59996337778863"/>
+        <fgColor theme="6" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519242"/>
+        <fgColor theme="6" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -703,19 +703,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79995117038484"/>
+        <fgColor theme="7" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59996337778863"/>
+        <fgColor theme="7" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519242"/>
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -726,19 +726,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79995117038484"/>
+        <fgColor theme="8" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59996337778863"/>
+        <fgColor theme="8" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519242"/>
+        <fgColor theme="8" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
@@ -749,24 +749,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79995117038484"/>
+        <fgColor theme="9" tint="0.79995117038483843"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59996337778863"/>
+        <fgColor theme="9" tint="0.59996337778862885"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519242"/>
+        <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -788,7 +788,7 @@
       <right/>
       <top/>
       <bottom style="thick">
-        <color theme="4" tint="0.49995422223579"/>
+        <color theme="4" tint="0.49995422223578601"/>
       </bottom>
       <diagonal/>
     </border>
@@ -797,7 +797,7 @@
       <right/>
       <top/>
       <bottom style="medium">
-        <color theme="4" tint="0.39997558519242"/>
+        <color theme="4" tint="0.39997558519241921"/>
       </bottom>
       <diagonal/>
     </border>
@@ -881,193 +881,191 @@
       </bottom>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="false" applyFont="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="false" applyFill="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="false" applyFill="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
-      <alignment vertical="center" wrapText="true"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="true" applyAlignment="true">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="true"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
-    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="true"/>
-    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="true"/>
-    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="true"/>
-    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="true"/>
-    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="true"/>
-    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="true"/>
-    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="true"/>
-    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="true"/>
-    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="true"/>
-    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="true"/>
-    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="true"/>
-    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="true"/>
-    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="true"/>
-    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="true"/>
-    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="true"/>
-    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="true"/>
-    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="true"/>
-    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="true"/>
-    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="true"/>
-    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="true"/>
-    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="true"/>
-    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="true"/>
-    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="true"/>
-    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="true"/>
-    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="true"/>
-    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="true"/>
-    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="true"/>
-    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="true"/>
-    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="true"/>
-    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="true"/>
-    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="true"/>
+    <cellStyle name="20% - 강조색1" xfId="19" builtinId="30" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색2" xfId="23" builtinId="34" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색3" xfId="27" builtinId="38" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색4" xfId="31" builtinId="42" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색5" xfId="35" builtinId="46" customBuiltin="1"/>
+    <cellStyle name="20% - 강조색6" xfId="39" builtinId="50" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색1" xfId="20" builtinId="31" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색2" xfId="24" builtinId="35" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색3" xfId="28" builtinId="39" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색4" xfId="32" builtinId="43" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색5" xfId="36" builtinId="47" customBuiltin="1"/>
+    <cellStyle name="40% - 강조색6" xfId="40" builtinId="51" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색1" xfId="21" builtinId="32" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색2" xfId="25" builtinId="36" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색3" xfId="29" builtinId="40" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색4" xfId="33" builtinId="44" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색5" xfId="37" builtinId="48" customBuiltin="1"/>
+    <cellStyle name="60% - 강조색6" xfId="41" builtinId="52" customBuiltin="1"/>
+    <cellStyle name="강조색1" xfId="18" builtinId="29" customBuiltin="1"/>
+    <cellStyle name="강조색2" xfId="22" builtinId="33" customBuiltin="1"/>
+    <cellStyle name="강조색3" xfId="26" builtinId="37" customBuiltin="1"/>
+    <cellStyle name="강조색4" xfId="30" builtinId="41" customBuiltin="1"/>
+    <cellStyle name="강조색5" xfId="34" builtinId="45" customBuiltin="1"/>
+    <cellStyle name="강조색6" xfId="38" builtinId="49" customBuiltin="1"/>
+    <cellStyle name="경고문" xfId="14" builtinId="11" customBuiltin="1"/>
+    <cellStyle name="계산" xfId="11" builtinId="22" customBuiltin="1"/>
+    <cellStyle name="나쁨" xfId="7" builtinId="27" customBuiltin="1"/>
+    <cellStyle name="메모" xfId="15" builtinId="10" customBuiltin="1"/>
+    <cellStyle name="보통" xfId="8" builtinId="28" customBuiltin="1"/>
+    <cellStyle name="설명 텍스트" xfId="16" builtinId="53" customBuiltin="1"/>
+    <cellStyle name="셀 확인" xfId="13" builtinId="23" customBuiltin="1"/>
+    <cellStyle name="연결된 셀" xfId="12" builtinId="24" customBuiltin="1"/>
+    <cellStyle name="요약" xfId="17" builtinId="25" customBuiltin="1"/>
+    <cellStyle name="입력" xfId="9" builtinId="20" customBuiltin="1"/>
+    <cellStyle name="제목" xfId="1" builtinId="15" customBuiltin="1"/>
+    <cellStyle name="제목 1" xfId="2" builtinId="16" customBuiltin="1"/>
+    <cellStyle name="제목 2" xfId="3" builtinId="17" customBuiltin="1"/>
+    <cellStyle name="제목 3" xfId="4" builtinId="18" customBuiltin="1"/>
+    <cellStyle name="제목 4" xfId="5" builtinId="19" customBuiltin="1"/>
+    <cellStyle name="좋음" xfId="6" builtinId="26" customBuiltin="1"/>
+    <cellStyle name="출력" xfId="10" builtinId="21" customBuiltin="1"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1084,7 +1082,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1235,7 +1233,7 @@
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1259,9 +1257,9 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1285,7 +1283,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1320,7 +1318,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="false">
+            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="63000"/>
               </a:srgbClr>
@@ -1338,7 +1336,7 @@
             <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="true">
+        <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
@@ -1363,7 +1361,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="false"/>
+          <a:lin ang="5400000" scaled="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
@@ -1379,673 +1377,444 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:U17"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.75" customWidth="true"/>
-    <col min="2" max="2" width="10" customWidth="true"/>
-    <col min="3" max="3" width="22.75" customWidth="true"/>
-    <col min="4" max="4" width="4" customWidth="true"/>
-    <col min="5" max="5" width="13.5" customWidth="true"/>
-    <col min="6" max="6" width="6.875" customWidth="true"/>
-    <col min="7" max="7" width="4.125" customWidth="true"/>
-    <col min="8" max="8" width="4" customWidth="true"/>
-    <col min="9" max="9" width="3.875" customWidth="true"/>
-    <col min="10" max="10" width="7.5" customWidth="true"/>
-    <col min="11" max="11" width="14.375" customWidth="true"/>
-    <col min="12" max="12" width="9.25" customWidth="true"/>
-    <col min="13" max="13" width="11" customWidth="true"/>
-    <col min="14" max="14" width="4.625" customWidth="true"/>
-    <col min="15" max="15" width="10.625" customWidth="true"/>
-    <col min="16" max="16" width="14.125" customWidth="true"/>
-    <col min="17" max="17" width="15.75" customWidth="true"/>
-    <col min="18" max="18" width="14.875" customWidth="true"/>
-    <col min="19" max="19" width="10.625" customWidth="true"/>
-    <col min="20" max="20" width="12.875" customWidth="true"/>
-    <col min="21" max="21" width="9.5" customWidth="true"/>
+    <col min="1" max="1" width="25.75" customWidth="1"/>
+    <col min="2" max="2" width="10.75" customWidth="1"/>
+    <col min="3" max="3" width="34.5" customWidth="1"/>
+    <col min="4" max="4" width="4" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="6.875" customWidth="1"/>
+    <col min="7" max="7" width="4.125" customWidth="1"/>
+    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="9" max="9" width="3.875" customWidth="1"/>
+    <col min="10" max="10" width="7.5" customWidth="1"/>
+    <col min="11" max="11" width="14.375" customWidth="1"/>
+    <col min="12" max="12" width="9.25" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="4.625" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
+    <col min="16" max="16" width="14.125" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.875" customWidth="1"/>
+    <col min="19" max="19" width="10.625" customWidth="1"/>
+    <col min="20" max="20" width="12.875" customWidth="1"/>
+    <col min="21" max="21" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B1" s="2">
         <v>0.01</v>
       </c>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
-      <c r="M1" s="0"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
-      <c r="P1" s="0"/>
-      <c r="Q1" s="0"/>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
-      <c r="T1" s="0"/>
-      <c r="U1" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>30</v>
       </c>
       <c r="B2" s="2">
         <v>0</v>
       </c>
-      <c r="C2" s="0"/>
-      <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
-      <c r="G2" s="0"/>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0"/>
-      <c r="K2" s="0"/>
-      <c r="L2" s="0"/>
-      <c r="M2" s="0"/>
-      <c r="N2" s="0"/>
-      <c r="O2" s="0"/>
-      <c r="P2" s="0"/>
-      <c r="Q2" s="0"/>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0"/>
-      <c r="T2" s="0"/>
-      <c r="U2" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>31</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
       </c>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="0"/>
-      <c r="O3" s="0"/>
-      <c r="P3" s="0"/>
-      <c r="Q3" s="0"/>
-      <c r="R3" s="0"/>
-      <c r="S3" s="0"/>
-      <c r="T3" s="0"/>
-      <c r="U3" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B4" s="2">
-        <v>0.029999999999999999</v>
-      </c>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
-      <c r="N4" s="0"/>
-      <c r="O4" s="0"/>
-      <c r="P4" s="0"/>
-      <c r="Q4" s="0"/>
-      <c r="R4" s="0"/>
-      <c r="S4" s="0"/>
-      <c r="T4" s="0"/>
-      <c r="U4" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="C5" s="0"/>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="0"/>
-      <c r="O5" s="0"/>
-      <c r="P5" s="0"/>
-      <c r="Q5" s="0"/>
-      <c r="R5" s="0"/>
-      <c r="S5" s="0"/>
-      <c r="T5" s="0"/>
-      <c r="U5" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
-      <c r="E6" s="0"/>
-      <c r="F6" s="0"/>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="0"/>
-      <c r="O6" s="0"/>
-      <c r="P6" s="0"/>
-      <c r="Q6" s="0"/>
-      <c r="R6" s="0"/>
-      <c r="S6" s="0"/>
-      <c r="T6" s="0"/>
-      <c r="U6" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>35</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
-      <c r="F7" s="0"/>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0"/>
-      <c r="K7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="0"/>
-      <c r="O7" s="0"/>
-      <c r="P7" s="0"/>
-      <c r="Q7" s="0"/>
-      <c r="R7" s="0"/>
-      <c r="S7" s="0"/>
-      <c r="T7" s="0"/>
-      <c r="U7" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" ht="165" x14ac:dyDescent="0.3">
+    </row>
+    <row r="8" spans="1:21" ht="165" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B8" s="2"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
-      <c r="O8" s="0"/>
-      <c r="P8" s="0"/>
-      <c r="Q8" s="0"/>
-      <c r="R8" s="0"/>
-      <c r="S8" s="0"/>
-      <c r="T8" s="0"/>
-      <c r="U8" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B9" s="2"/>
-      <c r="C9" s="0"/>
-      <c r="D9" s="0"/>
-      <c r="E9" s="0"/>
-      <c r="F9" s="0"/>
-      <c r="G9" s="0"/>
-      <c r="H9" s="0"/>
-      <c r="I9" s="0"/>
-      <c r="J9" s="0"/>
-      <c r="K9" s="0"/>
-      <c r="L9" s="0"/>
-      <c r="M9" s="0"/>
-      <c r="N9" s="0"/>
-      <c r="O9" s="0"/>
-      <c r="P9" s="0"/>
-      <c r="Q9" s="0"/>
-      <c r="R9" s="0"/>
-      <c r="S9" s="0"/>
-      <c r="T9" s="0"/>
-      <c r="U9" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>7</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" t="s">
         <v>8</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" t="s">
         <v>9</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" t="s">
         <v>10</v>
       </c>
-      <c r="G10" s="0" t="s">
+      <c r="G10" t="s">
         <v>11</v>
       </c>
-      <c r="H10" s="0" t="s">
+      <c r="H10" t="s">
         <v>12</v>
       </c>
-      <c r="I10" s="0" t="s">
+      <c r="I10" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="0" t="s">
+      <c r="J10" t="s">
         <v>14</v>
       </c>
-      <c r="K10" s="0" t="s">
+      <c r="K10" t="s">
         <v>15</v>
       </c>
-      <c r="L10" s="0" t="s">
+      <c r="L10" t="s">
         <v>16</v>
       </c>
-      <c r="M10" s="0" t="s">
+      <c r="M10" t="s">
         <v>17</v>
       </c>
-      <c r="N10" s="0" t="s">
+      <c r="N10" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="0" t="s">
+      <c r="O10" t="s">
         <v>19</v>
       </c>
-      <c r="P10" s="0" t="s">
+      <c r="P10" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" s="0" t="s">
+      <c r="Q10" t="s">
         <v>21</v>
       </c>
-      <c r="R10" s="0" t="s">
+      <c r="R10" t="s">
         <v>22</v>
       </c>
-      <c r="S10" s="0" t="s">
+      <c r="S10" t="s">
         <v>23</v>
       </c>
-      <c r="T10" s="0" t="s">
+      <c r="T10" t="s">
         <v>24</v>
       </c>
-      <c r="U10" s="0" t="s">
+      <c r="U10" t="s">
         <v>25</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
-      <c r="A11" s="0" t="s">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>99</v>
       </c>
-      <c r="B11" s="0">
+      <c r="B11">
         <v>260515</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>100</v>
       </c>
-      <c r="D11" s="0">
+      <c r="D11">
         <v>3</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" t="s">
         <v>73</v>
       </c>
-      <c r="F11" s="0"/>
-      <c r="G11" s="0"/>
-      <c r="H11" s="0"/>
-      <c r="I11" s="0"/>
-      <c r="J11" s="0"/>
-      <c r="K11" s="0" t="s">
+      <c r="K11" t="s">
         <v>99</v>
       </c>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
-      <c r="O11" s="0">
-        <v>1</v>
-      </c>
-      <c r="P11" s="0">
-        <v>0.010999999999999999</v>
-      </c>
-      <c r="Q11" s="0" t="s">
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>1.0999999999999999E-2</v>
+      </c>
+      <c r="Q11" t="s">
         <v>79</v>
       </c>
-      <c r="R11" s="0" t="s">
+      <c r="R11" t="s">
         <v>80</v>
       </c>
-      <c r="S11" s="0" t="s">
+      <c r="S11" t="s">
         <v>84</v>
       </c>
-      <c r="T11" s="0"/>
-      <c r="U11" s="0">
+      <c r="U11">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
-      <c r="A12" s="0" t="s">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="0">
+      <c r="B12">
         <v>260515</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>102</v>
       </c>
-      <c r="D12" s="0">
+      <c r="D12">
         <v>3</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" t="s">
         <v>73</v>
       </c>
-      <c r="F12" s="0"/>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
-      <c r="I12" s="0"/>
-      <c r="J12" s="0"/>
-      <c r="K12" s="0" t="s">
+      <c r="K12" t="s">
         <v>101</v>
       </c>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
-      <c r="O12" s="0">
-        <v>1</v>
-      </c>
-      <c r="P12" s="0">
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
         <v>0.70099999999999996</v>
       </c>
-      <c r="Q12" s="0" t="s">
+      <c r="Q12" t="s">
         <v>79</v>
       </c>
-      <c r="R12" s="0" t="s">
+      <c r="R12" t="s">
         <v>80</v>
       </c>
-      <c r="S12" s="0" t="s">
+      <c r="S12" t="s">
         <v>84</v>
       </c>
-      <c r="T12" s="0"/>
-      <c r="U12" s="0">
+      <c r="U12">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
-      <c r="A13" s="0" t="s">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="0">
+      <c r="B13">
         <v>260515</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>104</v>
       </c>
-      <c r="D13" s="0">
+      <c r="D13">
         <v>3</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0" t="s">
+      <c r="K13" t="s">
         <v>103</v>
       </c>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="0"/>
-      <c r="O13" s="0">
-        <v>1</v>
-      </c>
-      <c r="P13" s="0">
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
         <v>0.10100000000000001</v>
       </c>
-      <c r="Q13" s="0" t="s">
+      <c r="Q13" t="s">
         <v>79</v>
       </c>
-      <c r="R13" s="0" t="s">
+      <c r="R13" t="s">
         <v>80</v>
       </c>
-      <c r="S13" s="0" t="s">
+      <c r="S13" t="s">
         <v>84</v>
       </c>
-      <c r="T13" s="0"/>
-      <c r="U13" s="0">
+      <c r="U13">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
-      <c r="A14" s="0" t="s">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>105</v>
       </c>
-      <c r="B14" s="0">
+      <c r="B14">
         <v>260515</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>106</v>
       </c>
-      <c r="D14" s="0">
+      <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0" t="s">
+      <c r="K14" t="s">
         <v>105</v>
       </c>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="0"/>
-      <c r="O14" s="0">
-        <v>1</v>
-      </c>
-      <c r="P14" s="0">
-        <v>0.050999999999999997</v>
-      </c>
-      <c r="Q14" s="0" t="s">
+      <c r="O14">
+        <v>1</v>
+      </c>
+      <c r="P14">
+        <v>5.0999999999999997E-2</v>
+      </c>
+      <c r="Q14" t="s">
         <v>79</v>
       </c>
-      <c r="R14" s="0" t="s">
+      <c r="R14" t="s">
         <v>80</v>
       </c>
-      <c r="S14" s="0" t="s">
+      <c r="S14" t="s">
         <v>84</v>
       </c>
-      <c r="T14" s="0"/>
-      <c r="U14" s="0">
+      <c r="U14">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
-      <c r="A15" s="0" t="s">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>107</v>
       </c>
-      <c r="B15" s="0">
+      <c r="B15">
         <v>260515</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="0">
+      <c r="D15">
         <v>3</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" t="s">
         <v>73</v>
       </c>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0" t="s">
+      <c r="K15" t="s">
         <v>107</v>
       </c>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0">
-        <v>1</v>
-      </c>
-      <c r="P15" s="0">
+      <c r="O15">
+        <v>1</v>
+      </c>
+      <c r="P15">
         <v>1.0049999999999999</v>
       </c>
-      <c r="Q15" s="0" t="s">
+      <c r="Q15" t="s">
         <v>79</v>
       </c>
-      <c r="R15" s="0" t="s">
+      <c r="R15" t="s">
         <v>80</v>
       </c>
-      <c r="S15" s="0" t="s">
+      <c r="S15" t="s">
         <v>84</v>
       </c>
-      <c r="T15" s="0"/>
-      <c r="U15" s="0">
+      <c r="U15">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
-      <c r="A16" s="0" t="s">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="0">
+      <c r="B16">
         <v>260515</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>109</v>
       </c>
-      <c r="D16" s="0">
+      <c r="D16">
         <v>3</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>73</v>
       </c>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="K16" s="0" t="s">
+      <c r="K16" t="s">
         <v>108</v>
       </c>
-      <c r="L16" s="0"/>
-      <c r="M16" s="0"/>
-      <c r="N16" s="0"/>
-      <c r="O16" s="0">
-        <v>1</v>
-      </c>
-      <c r="P16" s="0">
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
         <v>2.0049999999999999</v>
       </c>
-      <c r="Q16" s="0" t="s">
+      <c r="Q16" t="s">
         <v>79</v>
       </c>
-      <c r="R16" s="0" t="s">
+      <c r="R16" t="s">
         <v>80</v>
       </c>
-      <c r="S16" s="0" t="s">
+      <c r="S16" t="s">
         <v>84</v>
       </c>
-      <c r="T16" s="0"/>
-      <c r="U16" s="0">
+      <c r="U16">
         <v>-1</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
-      <c r="A17" s="0" t="s">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>111</v>
       </c>
-      <c r="B17" s="0">
+      <c r="B17">
         <v>260615</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>95</v>
       </c>
-      <c r="D17" s="0">
+      <c r="D17">
         <v>3</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" t="s">
         <v>78</v>
       </c>
-      <c r="F17" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="G17" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="H17" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="I17" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="J17" s="0">
-        <v>1</v>
-      </c>
-      <c r="K17" s="0" t="s">
+      <c r="F17">
+        <v>0.1</v>
+      </c>
+      <c r="G17">
+        <v>0.1</v>
+      </c>
+      <c r="H17">
+        <v>0.1</v>
+      </c>
+      <c r="I17">
+        <v>0.1</v>
+      </c>
+      <c r="J17">
+        <v>1</v>
+      </c>
+      <c r="K17" t="s">
         <v>111</v>
       </c>
-      <c r="L17" s="0"/>
-      <c r="M17" s="0"/>
-      <c r="N17" s="0"/>
-      <c r="O17" s="0">
-        <v>1</v>
-      </c>
-      <c r="P17" s="0">
-        <v>0.001</v>
-      </c>
-      <c r="Q17" s="0" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>1E-3</v>
+      </c>
+      <c r="Q17" t="s">
         <v>74</v>
       </c>
-      <c r="R17" s="0" t="s">
+      <c r="R17" t="s">
         <v>28</v>
       </c>
-      <c r="S17" s="0" t="s">
+      <c r="S17" t="s">
         <v>75</v>
       </c>
-      <c r="T17" s="0"/>
-      <c r="U17" s="0">
+      <c r="U17">
         <v>-1</v>
       </c>
     </row>
@@ -2057,944 +1826,686 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BFFA8AF3-BD89-432D-8740-30DBF5179C15}">
   <dimension ref="A1:U22"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.375" customWidth="true"/>
-    <col min="2" max="2" width="7.25" customWidth="true"/>
-    <col min="3" max="3" width="24.75" customWidth="true"/>
-    <col min="4" max="4" width="4" customWidth="true"/>
-    <col min="5" max="5" width="13.5" customWidth="true"/>
-    <col min="6" max="6" width="6.875" customWidth="true"/>
-    <col min="7" max="7" width="4.125" customWidth="true"/>
-    <col min="8" max="8" width="4" customWidth="true"/>
-    <col min="9" max="9" width="3.875" customWidth="true"/>
-    <col min="10" max="10" width="7.5" customWidth="true"/>
-    <col min="11" max="11" width="11.375" customWidth="true"/>
-    <col min="12" max="12" width="9.25" customWidth="true"/>
-    <col min="13" max="13" width="11" customWidth="true"/>
-    <col min="14" max="14" width="4.625" customWidth="true"/>
-    <col min="15" max="15" width="10.625" customWidth="true"/>
-    <col min="16" max="16" width="14.125" customWidth="true"/>
-    <col min="17" max="17" width="15.75" customWidth="true"/>
-    <col min="18" max="18" width="14.875" customWidth="true"/>
-    <col min="19" max="19" width="10.625" customWidth="true"/>
-    <col min="20" max="20" width="12.875" customWidth="true"/>
-    <col min="21" max="21" width="9.5" customWidth="true"/>
+    <col min="1" max="1" width="10.375" customWidth="1"/>
+    <col min="2" max="2" width="7.25" customWidth="1"/>
+    <col min="3" max="3" width="24.75" customWidth="1"/>
+    <col min="4" max="4" width="4" customWidth="1"/>
+    <col min="5" max="5" width="13.5" customWidth="1"/>
+    <col min="6" max="6" width="6.875" customWidth="1"/>
+    <col min="7" max="7" width="4.125" customWidth="1"/>
+    <col min="8" max="8" width="4" customWidth="1"/>
+    <col min="9" max="9" width="3.875" customWidth="1"/>
+    <col min="10" max="10" width="7.5" customWidth="1"/>
+    <col min="11" max="11" width="11.375" customWidth="1"/>
+    <col min="12" max="12" width="9.25" customWidth="1"/>
+    <col min="13" max="13" width="11" customWidth="1"/>
+    <col min="14" max="14" width="4.625" customWidth="1"/>
+    <col min="15" max="15" width="10.625" customWidth="1"/>
+    <col min="16" max="16" width="14.125" customWidth="1"/>
+    <col min="17" max="17" width="15.75" customWidth="1"/>
+    <col min="18" max="18" width="14.875" customWidth="1"/>
+    <col min="19" max="19" width="10.625" customWidth="1"/>
+    <col min="20" max="20" width="12.875" customWidth="1"/>
+    <col min="21" max="21" width="9.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="0" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0">
-        <v>1</v>
-      </c>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
-      <c r="G1" s="0"/>
-      <c r="H1" s="0"/>
-      <c r="I1" s="0"/>
-      <c r="J1" s="0"/>
-      <c r="K1" s="0"/>
-      <c r="L1" s="0"/>
-      <c r="M1" s="0"/>
-      <c r="N1" s="0"/>
-      <c r="O1" s="0"/>
-      <c r="P1" s="0"/>
-      <c r="Q1" s="0"/>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
-      <c r="T1" s="0"/>
-      <c r="U1" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
-      <c r="A2" s="0" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="0">
+      <c r="B1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2">
         <v>0</v>
       </c>
-      <c r="C2" s="0"/>
-      <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
-      <c r="G2" s="0"/>
-      <c r="H2" s="0"/>
-      <c r="I2" s="0"/>
-      <c r="J2" s="0"/>
-      <c r="K2" s="0"/>
-      <c r="L2" s="0"/>
-      <c r="M2" s="0"/>
-      <c r="N2" s="0"/>
-      <c r="O2" s="0"/>
-      <c r="P2" s="0"/>
-      <c r="Q2" s="0"/>
-      <c r="R2" s="0"/>
-      <c r="S2" s="0"/>
-      <c r="T2" s="0"/>
-      <c r="U2" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
-      <c r="A3" s="0" t="s">
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="0">
+      <c r="B3">
         <v>0</v>
       </c>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
-      <c r="G3" s="0"/>
-      <c r="H3" s="0"/>
-      <c r="I3" s="0"/>
-      <c r="J3" s="0"/>
-      <c r="K3" s="0"/>
-      <c r="L3" s="0"/>
-      <c r="M3" s="0"/>
-      <c r="N3" s="0"/>
-      <c r="O3" s="0"/>
-      <c r="P3" s="0"/>
-      <c r="Q3" s="0"/>
-      <c r="R3" s="0"/>
-      <c r="S3" s="0"/>
-      <c r="T3" s="0"/>
-      <c r="U3" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
-      <c r="A4" s="0" t="s">
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="0">
+      <c r="B4">
         <v>0</v>
       </c>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
-      <c r="G4" s="0"/>
-      <c r="H4" s="0"/>
-      <c r="I4" s="0"/>
-      <c r="J4" s="0"/>
-      <c r="K4" s="0"/>
-      <c r="L4" s="0"/>
-      <c r="M4" s="0"/>
-      <c r="N4" s="0"/>
-      <c r="O4" s="0"/>
-      <c r="P4" s="0"/>
-      <c r="Q4" s="0"/>
-      <c r="R4" s="0"/>
-      <c r="S4" s="0"/>
-      <c r="T4" s="0"/>
-      <c r="U4" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
-      <c r="A5" s="0" t="s">
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="0">
+      <c r="B5">
         <v>0</v>
       </c>
-      <c r="C5" s="0"/>
-      <c r="D5" s="0"/>
-      <c r="E5" s="0"/>
-      <c r="F5" s="0"/>
-      <c r="G5" s="0"/>
-      <c r="H5" s="0"/>
-      <c r="I5" s="0"/>
-      <c r="J5" s="0"/>
-      <c r="K5" s="0"/>
-      <c r="L5" s="0"/>
-      <c r="M5" s="0"/>
-      <c r="N5" s="0"/>
-      <c r="O5" s="0"/>
-      <c r="P5" s="0"/>
-      <c r="Q5" s="0"/>
-      <c r="R5" s="0"/>
-      <c r="S5" s="0"/>
-      <c r="T5" s="0"/>
-      <c r="U5" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
-      <c r="A6" s="0" t="s">
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="0">
+      <c r="B6">
         <v>0</v>
       </c>
-      <c r="C6" s="0"/>
-      <c r="D6" s="0"/>
-      <c r="E6" s="0"/>
-      <c r="F6" s="0"/>
-      <c r="G6" s="0"/>
-      <c r="H6" s="0"/>
-      <c r="I6" s="0"/>
-      <c r="J6" s="0"/>
-      <c r="K6" s="0"/>
-      <c r="L6" s="0"/>
-      <c r="M6" s="0"/>
-      <c r="N6" s="0"/>
-      <c r="O6" s="0"/>
-      <c r="P6" s="0"/>
-      <c r="Q6" s="0"/>
-      <c r="R6" s="0"/>
-      <c r="S6" s="0"/>
-      <c r="T6" s="0"/>
-      <c r="U6" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
-      <c r="A7" s="0" t="s">
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="0">
-        <v>1</v>
-      </c>
-      <c r="C7" s="0"/>
-      <c r="D7" s="0"/>
-      <c r="E7" s="0"/>
-      <c r="F7" s="0"/>
-      <c r="G7" s="0"/>
-      <c r="H7" s="0"/>
-      <c r="I7" s="0"/>
-      <c r="J7" s="0"/>
-      <c r="K7" s="0"/>
-      <c r="L7" s="0"/>
-      <c r="M7" s="0"/>
-      <c r="N7" s="0"/>
-      <c r="O7" s="0"/>
-      <c r="P7" s="0"/>
-      <c r="Q7" s="0"/>
-      <c r="R7" s="0"/>
-      <c r="S7" s="0"/>
-      <c r="T7" s="0"/>
-      <c r="U7" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
-      <c r="A8" s="0" t="s">
+      <c r="B7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="0"/>
-      <c r="C8" s="0"/>
-      <c r="D8" s="0"/>
-      <c r="E8" s="0"/>
-      <c r="F8" s="0"/>
-      <c r="G8" s="0"/>
-      <c r="H8" s="0"/>
-      <c r="I8" s="0"/>
-      <c r="J8" s="0"/>
-      <c r="K8" s="0"/>
-      <c r="L8" s="0"/>
-      <c r="M8" s="0"/>
-      <c r="N8" s="0"/>
-      <c r="O8" s="0"/>
-      <c r="P8" s="0"/>
-      <c r="Q8" s="0"/>
-      <c r="R8" s="0"/>
-      <c r="S8" s="0"/>
-      <c r="T8" s="0"/>
-      <c r="U8" s="0"/>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
-      <c r="A9" s="0" t="s">
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" t="s">
         <v>7</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" t="s">
         <v>10</v>
       </c>
-      <c r="G9" s="0" t="s">
+      <c r="G9" t="s">
         <v>11</v>
       </c>
-      <c r="H9" s="0" t="s">
+      <c r="H9" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="0" t="s">
+      <c r="I9" t="s">
         <v>13</v>
       </c>
-      <c r="J9" s="0" t="s">
+      <c r="J9" t="s">
         <v>14</v>
       </c>
-      <c r="K9" s="0" t="s">
+      <c r="K9" t="s">
         <v>15</v>
       </c>
-      <c r="L9" s="0" t="s">
+      <c r="L9" t="s">
         <v>16</v>
       </c>
-      <c r="M9" s="0" t="s">
+      <c r="M9" t="s">
         <v>17</v>
       </c>
-      <c r="N9" s="0" t="s">
+      <c r="N9" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="0" t="s">
+      <c r="O9" t="s">
         <v>19</v>
       </c>
-      <c r="P9" s="0" t="s">
+      <c r="P9" t="s">
         <v>20</v>
       </c>
-      <c r="Q9" s="0" t="s">
+      <c r="Q9" t="s">
         <v>21</v>
       </c>
-      <c r="R9" s="0" t="s">
+      <c r="R9" t="s">
         <v>22</v>
       </c>
-      <c r="S9" s="0" t="s">
+      <c r="S9" t="s">
         <v>23</v>
       </c>
-      <c r="T9" s="0" t="s">
+      <c r="T9" t="s">
         <v>24</v>
       </c>
-      <c r="U9" s="0" t="s">
+      <c r="U9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
-      <c r="A10" s="0" t="s">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>77</v>
       </c>
-      <c r="B10" s="0">
+      <c r="B10">
         <v>260501</v>
       </c>
-      <c r="C10" s="0" t="s">
+      <c r="C10" t="s">
         <v>62</v>
       </c>
-      <c r="D10" s="0">
+      <c r="D10">
         <v>3</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" t="s">
         <v>78</v>
       </c>
-      <c r="F10" s="0">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="G10" s="0">
-        <v>0.29999999999999999</v>
-      </c>
-      <c r="H10" s="0">
+      <c r="F10">
+        <v>0.2</v>
+      </c>
+      <c r="G10">
+        <v>0.3</v>
+      </c>
+      <c r="H10">
         <v>0</v>
       </c>
-      <c r="I10" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="J10" s="0">
-        <v>1</v>
-      </c>
-      <c r="K10" s="0" t="s">
+      <c r="I10">
+        <v>0.1</v>
+      </c>
+      <c r="J10">
+        <v>1</v>
+      </c>
+      <c r="K10" t="s">
         <v>77</v>
       </c>
-      <c r="L10" s="0"/>
-      <c r="M10" s="0"/>
-      <c r="N10" s="0"/>
-      <c r="O10" s="0">
-        <v>1</v>
-      </c>
-      <c r="P10" s="0">
-        <v>0.0001</v>
-      </c>
-      <c r="Q10" s="0" t="s">
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="P10">
+        <v>1E-4</v>
+      </c>
+      <c r="Q10" t="s">
         <v>79</v>
       </c>
-      <c r="R10" s="0" t="s">
+      <c r="R10" t="s">
         <v>80</v>
       </c>
-      <c r="S10" s="0" t="s">
+      <c r="S10" t="s">
         <v>75</v>
       </c>
-      <c r="T10" s="0"/>
-      <c r="U10" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
-      <c r="A11" s="0" t="s">
+      <c r="U10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>81</v>
       </c>
-      <c r="B11" s="0">
+      <c r="B11">
         <v>260501</v>
       </c>
-      <c r="C11" s="0" t="s">
+      <c r="C11" t="s">
         <v>63</v>
       </c>
-      <c r="D11" s="0">
+      <c r="D11">
         <v>3</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" t="s">
         <v>78</v>
       </c>
-      <c r="F11" s="0">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="G11" s="0">
-        <v>0.29999999999999999</v>
-      </c>
-      <c r="H11" s="0">
+      <c r="F11">
+        <v>0.2</v>
+      </c>
+      <c r="G11">
+        <v>0.3</v>
+      </c>
+      <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="J11" s="0">
-        <v>1</v>
-      </c>
-      <c r="K11" s="0" t="s">
+      <c r="I11">
+        <v>0.1</v>
+      </c>
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s">
         <v>81</v>
       </c>
-      <c r="L11" s="0"/>
-      <c r="M11" s="0"/>
-      <c r="N11" s="0"/>
-      <c r="O11" s="0">
-        <v>1</v>
-      </c>
-      <c r="P11" s="0">
-        <v>0.0001</v>
-      </c>
-      <c r="Q11" s="0" t="s">
+      <c r="O11">
+        <v>1</v>
+      </c>
+      <c r="P11">
+        <v>1E-4</v>
+      </c>
+      <c r="Q11" t="s">
         <v>79</v>
       </c>
-      <c r="R11" s="0" t="s">
+      <c r="R11" t="s">
         <v>80</v>
       </c>
-      <c r="S11" s="0" t="s">
+      <c r="S11" t="s">
         <v>75</v>
       </c>
-      <c r="T11" s="0"/>
-      <c r="U11" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
-      <c r="A12" s="0" t="s">
+      <c r="U11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
         <v>82</v>
       </c>
-      <c r="B12" s="0">
+      <c r="B12">
         <v>260501</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="C12" t="s">
         <v>64</v>
       </c>
-      <c r="D12" s="0">
+      <c r="D12">
         <v>3</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" t="s">
         <v>78</v>
       </c>
-      <c r="F12" s="0">
-        <v>0.20000000000000001</v>
-      </c>
-      <c r="G12" s="0">
-        <v>0.29999999999999999</v>
-      </c>
-      <c r="H12" s="0">
+      <c r="F12">
+        <v>0.2</v>
+      </c>
+      <c r="G12">
+        <v>0.3</v>
+      </c>
+      <c r="H12">
         <v>0</v>
       </c>
-      <c r="I12" s="0">
-        <v>0.10000000000000001</v>
-      </c>
-      <c r="J12" s="0">
-        <v>1</v>
-      </c>
-      <c r="K12" s="0" t="s">
+      <c r="I12">
+        <v>0.1</v>
+      </c>
+      <c r="J12">
+        <v>1</v>
+      </c>
+      <c r="K12" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="0"/>
-      <c r="M12" s="0"/>
-      <c r="N12" s="0"/>
-      <c r="O12" s="0">
-        <v>1</v>
-      </c>
-      <c r="P12" s="0">
-        <v>0.0001</v>
-      </c>
-      <c r="Q12" s="0" t="s">
+      <c r="O12">
+        <v>1</v>
+      </c>
+      <c r="P12">
+        <v>1E-4</v>
+      </c>
+      <c r="Q12" t="s">
         <v>79</v>
       </c>
-      <c r="R12" s="0" t="s">
+      <c r="R12" t="s">
         <v>80</v>
       </c>
-      <c r="S12" s="0" t="s">
+      <c r="S12" t="s">
         <v>75</v>
       </c>
-      <c r="T12" s="0"/>
-      <c r="U12" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
-      <c r="A13" s="0" t="s">
+      <c r="U12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>83</v>
       </c>
-      <c r="B13" s="0">
+      <c r="B13">
         <v>260513</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="0">
+      <c r="D13">
         <v>3</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" t="s">
         <v>73</v>
       </c>
-      <c r="F13" s="0"/>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
-      <c r="I13" s="0"/>
-      <c r="J13" s="0"/>
-      <c r="K13" s="0" t="s">
+      <c r="K13" t="s">
         <v>83</v>
       </c>
-      <c r="L13" s="0"/>
-      <c r="M13" s="0"/>
-      <c r="N13" s="0"/>
-      <c r="O13" s="0"/>
-      <c r="P13" s="0"/>
-      <c r="Q13" s="0"/>
-      <c r="R13" s="0"/>
-      <c r="S13" s="0" t="s">
+      <c r="S13" t="s">
         <v>84</v>
       </c>
-      <c r="T13" s="0"/>
-      <c r="U13" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
-      <c r="A14" s="0" t="s">
+      <c r="U13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
         <v>85</v>
       </c>
-      <c r="B14" s="0">
+      <c r="B14">
         <v>260513</v>
       </c>
-      <c r="C14" s="0" t="s">
+      <c r="C14" t="s">
         <v>86</v>
       </c>
-      <c r="D14" s="0">
+      <c r="D14">
         <v>3</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" t="s">
         <v>73</v>
       </c>
-      <c r="F14" s="0"/>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
-      <c r="I14" s="0"/>
-      <c r="J14" s="0"/>
-      <c r="K14" s="0" t="s">
+      <c r="K14" t="s">
         <v>85</v>
       </c>
-      <c r="L14" s="0"/>
-      <c r="M14" s="0"/>
-      <c r="N14" s="0"/>
-      <c r="O14" s="0"/>
-      <c r="P14" s="0"/>
-      <c r="Q14" s="0"/>
-      <c r="R14" s="0"/>
-      <c r="S14" s="0" t="s">
+      <c r="S14" t="s">
         <v>84</v>
       </c>
-      <c r="T14" s="0"/>
-      <c r="U14" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
-      <c r="A15" s="0" t="s">
+      <c r="U14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
         <v>87</v>
       </c>
-      <c r="B15" s="0">
+      <c r="B15">
         <v>260513</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" t="s">
         <v>88</v>
       </c>
-      <c r="D15" s="0">
+      <c r="D15">
         <v>3</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" t="s">
         <v>73</v>
       </c>
-      <c r="F15" s="0"/>
-      <c r="G15" s="0"/>
-      <c r="H15" s="0"/>
-      <c r="I15" s="0"/>
-      <c r="J15" s="0"/>
-      <c r="K15" s="0" t="s">
+      <c r="K15" t="s">
         <v>87</v>
       </c>
-      <c r="L15" s="0"/>
-      <c r="M15" s="0"/>
-      <c r="N15" s="0"/>
-      <c r="O15" s="0"/>
-      <c r="P15" s="0"/>
-      <c r="Q15" s="0"/>
-      <c r="R15" s="0"/>
-      <c r="S15" s="0" t="s">
+      <c r="S15" t="s">
         <v>84</v>
       </c>
-      <c r="T15" s="0"/>
-      <c r="U15" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
-      <c r="A16" s="0" t="s">
+      <c r="U15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
         <v>89</v>
       </c>
-      <c r="B16" s="0">
+      <c r="B16">
         <v>260419</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="0">
+      <c r="D16">
         <v>3</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" t="s">
         <v>90</v>
       </c>
-      <c r="F16" s="0"/>
-      <c r="G16" s="0"/>
-      <c r="H16" s="0"/>
-      <c r="I16" s="0"/>
-      <c r="J16" s="0"/>
-      <c r="K16" s="0" t="s">
+      <c r="K16" t="s">
         <v>89</v>
       </c>
-      <c r="L16" s="0">
+      <c r="L16">
         <v>0.01</v>
       </c>
-      <c r="M16" s="0">
+      <c r="M16">
         <v>0</v>
       </c>
-      <c r="N16" s="0" t="s">
+      <c r="N16" t="s">
         <v>91</v>
       </c>
-      <c r="O16" s="0">
-        <v>1</v>
-      </c>
-      <c r="P16" s="0">
-        <v>0.001</v>
-      </c>
-      <c r="Q16" s="0" t="s">
+      <c r="O16">
+        <v>1</v>
+      </c>
+      <c r="P16">
+        <v>1E-3</v>
+      </c>
+      <c r="Q16" t="s">
         <v>74</v>
       </c>
-      <c r="R16" s="0" t="s">
+      <c r="R16" t="s">
         <v>28</v>
       </c>
-      <c r="S16" s="0" t="s">
+      <c r="S16" t="s">
         <v>75</v>
       </c>
-      <c r="T16" s="0"/>
-      <c r="U16" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
-      <c r="A17" s="0" t="s">
+      <c r="U16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
         <v>92</v>
       </c>
-      <c r="B17" s="0">
+      <c r="B17">
         <v>260419</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" t="s">
         <v>110</v>
       </c>
-      <c r="D17" s="0">
+      <c r="D17">
         <v>3</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" t="s">
         <v>90</v>
       </c>
-      <c r="F17" s="0"/>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
-      <c r="I17" s="0"/>
-      <c r="J17" s="0"/>
-      <c r="K17" s="0" t="s">
+      <c r="K17" t="s">
         <v>92</v>
       </c>
-      <c r="L17" s="0">
+      <c r="L17">
         <v>0.01</v>
       </c>
-      <c r="M17" s="0">
+      <c r="M17">
         <v>0</v>
       </c>
-      <c r="N17" s="0" t="s">
+      <c r="N17" t="s">
         <v>91</v>
       </c>
-      <c r="O17" s="0">
-        <v>1</v>
-      </c>
-      <c r="P17" s="0">
-        <v>0.0050000000000000001</v>
-      </c>
-      <c r="Q17" s="0" t="s">
+      <c r="O17">
+        <v>1</v>
+      </c>
+      <c r="P17">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="Q17" t="s">
         <v>74</v>
       </c>
-      <c r="R17" s="0" t="s">
+      <c r="R17" t="s">
         <v>28</v>
       </c>
-      <c r="S17" s="0" t="s">
+      <c r="S17" t="s">
         <v>75</v>
       </c>
-      <c r="T17" s="0"/>
-      <c r="U17" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
-      <c r="A18" s="0" t="s">
+      <c r="U17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>93</v>
       </c>
-      <c r="B18" s="0">
+      <c r="B18">
         <v>260419</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" t="s">
         <v>110</v>
       </c>
-      <c r="D18" s="0">
+      <c r="D18">
         <v>3</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" t="s">
         <v>90</v>
       </c>
-      <c r="F18" s="0"/>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0"/>
-      <c r="I18" s="0"/>
-      <c r="J18" s="0"/>
-      <c r="K18" s="0" t="s">
+      <c r="K18" t="s">
         <v>93</v>
       </c>
-      <c r="L18" s="0">
+      <c r="L18">
         <v>0.01</v>
       </c>
-      <c r="M18" s="0">
+      <c r="M18">
         <v>0</v>
       </c>
-      <c r="N18" s="0" t="s">
+      <c r="N18" t="s">
         <v>91</v>
       </c>
-      <c r="O18" s="0">
-        <v>1</v>
-      </c>
-      <c r="P18" s="0">
+      <c r="O18">
+        <v>1</v>
+      </c>
+      <c r="P18">
         <v>0.01</v>
       </c>
-      <c r="Q18" s="0" t="s">
+      <c r="Q18" t="s">
         <v>74</v>
       </c>
-      <c r="R18" s="0" t="s">
+      <c r="R18" t="s">
         <v>28</v>
       </c>
-      <c r="S18" s="0" t="s">
+      <c r="S18" t="s">
         <v>75</v>
       </c>
-      <c r="T18" s="0"/>
-      <c r="U18" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
-      <c r="A19" s="0" t="s">
+      <c r="U18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="0">
+      <c r="B19">
         <v>260416</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" t="s">
         <v>95</v>
       </c>
-      <c r="D19" s="0">
+      <c r="D19">
         <v>3</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" t="s">
         <v>73</v>
       </c>
-      <c r="F19" s="0"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
-      <c r="I19" s="0"/>
-      <c r="J19" s="0"/>
-      <c r="K19" s="0" t="s">
+      <c r="K19" t="s">
         <v>94</v>
       </c>
-      <c r="L19" s="0"/>
-      <c r="M19" s="0"/>
-      <c r="N19" s="0"/>
-      <c r="O19" s="0">
-        <v>1</v>
-      </c>
-      <c r="P19" s="0">
-        <v>0.001</v>
-      </c>
-      <c r="Q19" s="0" t="s">
+      <c r="O19">
+        <v>1</v>
+      </c>
+      <c r="P19">
+        <v>1E-3</v>
+      </c>
+      <c r="Q19" t="s">
         <v>74</v>
       </c>
-      <c r="R19" s="0" t="s">
+      <c r="R19" t="s">
         <v>28</v>
       </c>
-      <c r="S19" s="0" t="s">
+      <c r="S19" t="s">
         <v>75</v>
       </c>
-      <c r="T19" s="0"/>
-      <c r="U19" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
-      <c r="A20" s="0" t="s">
+      <c r="U19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>96</v>
       </c>
-      <c r="B20" s="0">
+      <c r="B20">
         <v>260416</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" t="s">
         <v>95</v>
       </c>
-      <c r="D20" s="0">
+      <c r="D20">
         <v>3</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" t="s">
         <v>73</v>
       </c>
-      <c r="F20" s="0"/>
-      <c r="G20" s="0"/>
-      <c r="H20" s="0"/>
-      <c r="I20" s="0"/>
-      <c r="J20" s="0"/>
-      <c r="K20" s="0" t="s">
+      <c r="K20" t="s">
         <v>96</v>
       </c>
-      <c r="L20" s="0"/>
-      <c r="M20" s="0"/>
-      <c r="N20" s="0"/>
-      <c r="O20" s="0">
-        <v>1</v>
-      </c>
-      <c r="P20" s="0">
-        <v>0.0050000000000000001</v>
-      </c>
-      <c r="Q20" s="0" t="s">
+      <c r="O20">
+        <v>1</v>
+      </c>
+      <c r="P20">
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="Q20" t="s">
         <v>74</v>
       </c>
-      <c r="R20" s="0" t="s">
+      <c r="R20" t="s">
         <v>28</v>
       </c>
-      <c r="S20" s="0" t="s">
+      <c r="S20" t="s">
         <v>75</v>
       </c>
-      <c r="T20" s="0"/>
-      <c r="U20" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
-      <c r="A21" s="0" t="s">
+      <c r="U20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>97</v>
       </c>
-      <c r="B21" s="0">
+      <c r="B21">
         <v>260416</v>
       </c>
-      <c r="C21" s="0" t="s">
+      <c r="C21" t="s">
         <v>95</v>
       </c>
-      <c r="D21" s="0">
+      <c r="D21">
         <v>3</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" t="s">
         <v>73</v>
       </c>
-      <c r="F21" s="0"/>
-      <c r="G21" s="0"/>
-      <c r="H21" s="0"/>
-      <c r="I21" s="0"/>
-      <c r="J21" s="0"/>
-      <c r="K21" s="0" t="s">
+      <c r="K21" t="s">
         <v>97</v>
       </c>
-      <c r="L21" s="0"/>
-      <c r="M21" s="0"/>
-      <c r="N21" s="0"/>
-      <c r="O21" s="0">
-        <v>1</v>
-      </c>
-      <c r="P21" s="0">
+      <c r="O21">
+        <v>1</v>
+      </c>
+      <c r="P21">
         <v>0.01</v>
       </c>
-      <c r="Q21" s="0" t="s">
+      <c r="Q21" t="s">
         <v>74</v>
       </c>
-      <c r="R21" s="0" t="s">
+      <c r="R21" t="s">
         <v>28</v>
       </c>
-      <c r="S21" s="0" t="s">
+      <c r="S21" t="s">
         <v>75</v>
       </c>
-      <c r="T21" s="0"/>
-      <c r="U21" s="0">
-        <v>1</v>
-      </c>
-    </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
-      <c r="A22" s="0" t="s">
+      <c r="U21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="0">
+      <c r="B22">
         <v>260416</v>
       </c>
-      <c r="C22" s="0" t="s">
+      <c r="C22" t="s">
         <v>95</v>
       </c>
-      <c r="D22" s="0">
+      <c r="D22">
         <v>3</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" t="s">
         <v>73</v>
       </c>
-      <c r="F22" s="0"/>
-      <c r="G22" s="0"/>
-      <c r="H22" s="0"/>
-      <c r="I22" s="0"/>
-      <c r="J22" s="0"/>
-      <c r="K22" s="0" t="s">
+      <c r="K22" t="s">
         <v>98</v>
       </c>
-      <c r="L22" s="0"/>
-      <c r="M22" s="0"/>
-      <c r="N22" s="0"/>
-      <c r="O22" s="0">
-        <v>1</v>
-      </c>
-      <c r="P22" s="0">
-        <v>0.029999999999999999</v>
-      </c>
-      <c r="Q22" s="0" t="s">
+      <c r="O22">
+        <v>1</v>
+      </c>
+      <c r="P22">
+        <v>0.03</v>
+      </c>
+      <c r="Q22" t="s">
         <v>74</v>
       </c>
-      <c r="R22" s="0" t="s">
+      <c r="R22" t="s">
         <v>28</v>
       </c>
-      <c r="S22" s="0" t="s">
+      <c r="S22" t="s">
         <v>75</v>
       </c>
-      <c r="T22" s="0"/>
-      <c r="U22" s="0">
+      <c r="U22">
         <v>1</v>
       </c>
     </row>
@@ -3006,20 +2517,20 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2D08ED25-9270-46EF-B411-03170886A4BC}">
   <dimension ref="A1:G30"/>
-  <sheetFormatPr xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.375" customWidth="true"/>
-    <col min="2" max="2" width="24.75" customWidth="true"/>
-    <col min="3" max="3" width="7.25" customWidth="true"/>
-    <col min="4" max="4" width="5.75" customWidth="true"/>
-    <col min="5" max="5" width="6.25" customWidth="true"/>
-    <col min="6" max="6" width="4" customWidth="true"/>
-    <col min="7" max="7" width="9.375" customWidth="true"/>
+    <col min="1" max="1" width="27.375" customWidth="1"/>
+    <col min="2" max="2" width="24.75" customWidth="1"/>
+    <col min="3" max="3" width="7.25" customWidth="1"/>
+    <col min="4" max="4" width="5.75" customWidth="1"/>
+    <col min="5" max="5" width="6.25" customWidth="1"/>
+    <col min="6" max="6" width="4" customWidth="1"/>
+    <col min="7" max="7" width="9.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -3027,7 +2538,7 @@
         <v>19</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>53</v>
       </c>
@@ -3035,7 +2546,7 @@
         <v>3</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>49</v>
       </c>
@@ -3043,12 +2554,12 @@
         <v>3</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>37</v>
       </c>
@@ -3071,7 +2582,7 @@
         <v>43</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>45</v>
       </c>
@@ -3088,7 +2599,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
@@ -3105,7 +2616,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -3122,7 +2633,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -3139,7 +2650,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>51</v>
       </c>
@@ -3156,7 +2667,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>52</v>
       </c>
@@ -3173,7 +2684,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>54</v>
       </c>
@@ -3190,7 +2701,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>55</v>
       </c>
@@ -3207,7 +2718,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>56</v>
       </c>
@@ -3224,7 +2735,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="15" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>57</v>
       </c>
@@ -3241,7 +2752,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>58</v>
       </c>
@@ -3258,7 +2769,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="17" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>59</v>
       </c>
@@ -3275,7 +2786,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="18" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>60</v>
       </c>
@@ -3292,7 +2803,7 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="19" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>61</v>
       </c>
@@ -3309,7 +2820,7 @@
         <v>1.05</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>62</v>
       </c>
@@ -3326,7 +2837,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="21" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -3343,7 +2854,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="22" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>64</v>
       </c>
@@ -3360,7 +2871,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="23" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>65</v>
       </c>
@@ -3377,7 +2888,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="24" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -3394,7 +2905,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>67</v>
       </c>
@@ -3411,7 +2922,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="26" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>68</v>
       </c>
@@ -3428,7 +2939,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="27" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>69</v>
       </c>
@@ -3445,7 +2956,7 @@
         <v>2</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="28" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -3462,7 +2973,7 @@
         <v>1.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="29" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>71</v>
       </c>
@@ -3479,7 +2990,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" r="30" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>72</v>
       </c>

</xml_diff>